<commit_message>
Tempo de reabsorção no cenário B (pior valor observado), cenário B-bio e η = 1
Permanentes recebem o pior valor observado (O2); B-bio só com os
bioabsorvíveis; sentinelas O1 e η passam a análise de sensibilidade.
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -21055,10 +21055,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
   </cols>
@@ -21105,7 +21105,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Inclui investigação e bioabsorvíveis (stent: A + Mg WE43 e PLLA)</t>
+          <t>Inclui investigação e bioabsorvíveis (stent: A + Mg WE43 e PLLA; permanentes com o pior valor observado no tempo de reabsorção, opção O2)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -21117,63 +21117,63 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>B-bio</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Só critérios quantitativos (sem ordinais)</t>
+          <t>Só bioabsorvíveis (Mg WE43 e PLLA) com o tempo de reabsorção; comparação, não ranking (opção O3)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Haste, stent, scaffold</t>
+          <t>Stent</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>R-sentinela</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sensibilidade dos pesos</t>
+          <t>Sensibilidade do tempo de reabsorção atribuído aos permanentes: 60, 120, 600 e 1200 meses (opção O1)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Todos os quantitativos</t>
+          <t>Stent</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>η</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nível de confiança</t>
+          <t>Só critérios quantitativos (sem ordinais)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Todos os quantitativos</t>
+          <t>Haste, stent, scaffold</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>W</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Concordância entre métodos</t>
+          <t>Sensibilidade dos pesos</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -21185,49 +21185,83 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>T-scaffold</t>
+          <t>η</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sensibilidade dos alvos</t>
+          <t>Sensibilidade ao nível de confiança η de 0 a 1, passo 0,1 (resultado principal: η = 1)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Scaffold</t>
+          <t>Todos os quantitativos</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T-haste</t>
+          <t>M</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sensibilidade do alvo de E (inclui 14 GPa, Petković et al. 2025, vs 17 GPa)</t>
+          <t>Concordância entre métodos</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Haste</t>
+          <t>Todos os quantitativos</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>T-scaffold</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Sensibilidade dos alvos</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Scaffold</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>T-haste</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sensibilidade do alvo de E (inclui 14 GPa, Petković et al. 2025, vs 17 GPa)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Haste</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>MC</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Incerteza das propriedades</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Todos os quantitativos</t>
         </is>
@@ -21622,11 +21656,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>η: confiança do decisor nos pesos subjetivos (0 = só pesos objetivos; 1 = só subjetivos); eq. 1 de Petković et al. 2025</t>
+          <t>η: confiança do decisor nos pesos subjetivos (0 = só objetivos; 1 = só subjetivos); eq. 1 de Petković et al. 2025. Resultado principal com η = 1; η de 0 a 1 só como sensibilidade</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Análise de robustez e run_all.py com todos os cenários de cenarios.csv
Monte Carlo de propriedades e pesos (n_iter configurável; 10 000, seed 42),
variantes Q, η, T-haste, T-scaffold, C-custo, R-sentinela e B-bio; resumo
por caso em results/resumo_robustez.md.
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -21055,7 +21055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -21253,15 +21253,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>C-custo</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Peso do custo relativo baixo (0,01) vs elevado (0,25), restantes pesos redistribuídos</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Todos os quantitativos</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>MC</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Incerteza das propriedades</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Todos os quantitativos</t>
         </is>

</xml_diff>

<commit_message>
Estatutos clínicos do scaffold (a confirmar) e resumo de robustez atualizado
Cenário A do scaffold passa a 5 materiais; reversão de ranking registada
nas notas metodológicas.
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -9498,7 +9498,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -9524,7 +9524,7 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
         </is>
       </c>
       <c r="N139" t="n">
@@ -9564,7 +9564,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -9590,7 +9590,7 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
         </is>
       </c>
       <c r="N140" t="n">
@@ -9630,7 +9630,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -9654,6 +9654,11 @@
           <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
         </is>
       </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+        </is>
+      </c>
       <c r="N141" t="n">
         <v>65</v>
       </c>
@@ -9691,7 +9696,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -9715,6 +9720,11 @@
           <t>Woodruff MA, Hutmacher DW. Prog Polym Sci 2010;35:1217-1256 (PCL)</t>
         </is>
       </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+        </is>
+      </c>
       <c r="N142" t="n">
         <v>30</v>
       </c>
@@ -9752,7 +9762,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -9776,6 +9786,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+        </is>
+      </c>
       <c r="N143" t="n">
         <v>1</v>
       </c>
@@ -9813,7 +9828,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -9837,6 +9852,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+        </is>
+      </c>
       <c r="N144" t="n">
         <v>5</v>
       </c>
@@ -9874,7 +9894,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -9900,7 +9920,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N145" t="n">
@@ -9940,7 +9960,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -9966,7 +9986,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N146" t="n">
@@ -10006,7 +10026,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -10030,6 +10050,11 @@
           <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
         </is>
       </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+        </is>
+      </c>
       <c r="N147" t="n">
         <v>75</v>
       </c>
@@ -10067,7 +10092,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -10091,6 +10116,11 @@
           <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
         </is>
       </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+        </is>
+      </c>
       <c r="N148" t="n">
         <v>27</v>
       </c>
@@ -10128,7 +10158,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -10152,6 +10182,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+        </is>
+      </c>
       <c r="N149" t="n">
         <v>1</v>
       </c>
@@ -10189,7 +10224,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -10213,6 +10248,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+        </is>
+      </c>
       <c r="N150" t="n">
         <v>4</v>
       </c>
@@ -10250,7 +10290,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -10276,7 +10316,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
         </is>
       </c>
       <c r="N151" t="n">
@@ -10316,7 +10356,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -10342,7 +10382,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
         </is>
       </c>
       <c r="N152" t="n">
@@ -10382,7 +10422,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -10406,6 +10446,11 @@
           <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
         </is>
       </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+        </is>
+      </c>
       <c r="N153" t="n">
         <v>80</v>
       </c>
@@ -10443,7 +10488,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -10467,6 +10512,11 @@
           <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
         </is>
       </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+        </is>
+      </c>
       <c r="N154" t="n">
         <v>2</v>
       </c>
@@ -10504,7 +10554,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -10528,6 +10578,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+        </is>
+      </c>
       <c r="N155" t="n">
         <v>1</v>
       </c>
@@ -10565,7 +10620,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -10589,6 +10644,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+        </is>
+      </c>
       <c r="N156" t="n">
         <v>3</v>
       </c>
@@ -10626,7 +10686,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -10652,7 +10712,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N157" t="n">
@@ -10692,7 +10752,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -10718,7 +10778,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N158" t="n">
@@ -10758,7 +10818,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -10782,6 +10842,11 @@
           <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
         </is>
       </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N159" t="n">
         <v>65</v>
       </c>
@@ -10819,7 +10884,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -10843,6 +10908,11 @@
           <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
         </is>
       </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N160" t="n">
         <v>42</v>
       </c>
@@ -10880,7 +10950,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -10904,6 +10974,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N161" t="n">
         <v>4</v>
       </c>
@@ -10941,7 +11016,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -10965,6 +11040,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N162" t="n">
         <v>2</v>
       </c>
@@ -11002,7 +11082,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -11028,7 +11108,7 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N163" t="n">
@@ -11068,7 +11148,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -11094,7 +11174,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N164" t="n">
@@ -11134,7 +11214,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -11158,6 +11238,11 @@
           <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
         </is>
       </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N165" t="n">
         <v>65</v>
       </c>
@@ -11195,7 +11280,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -11219,6 +11304,11 @@
           <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
         </is>
       </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N166" t="n">
         <v>12</v>
       </c>
@@ -11256,7 +11346,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -11280,6 +11370,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N167" t="n">
         <v>4</v>
       </c>
@@ -11317,7 +11412,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -11341,6 +11436,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N168" t="n">
         <v>2</v>
       </c>
@@ -11378,7 +11478,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -11404,7 +11504,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
         </is>
       </c>
       <c r="N169" t="n">
@@ -11444,7 +11544,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -11470,7 +11570,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
         </is>
       </c>
       <c r="N170" t="n">
@@ -11510,7 +11610,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -11534,6 +11634,11 @@
           <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
         </is>
       </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+        </is>
+      </c>
       <c r="N171" t="n">
         <v>80</v>
       </c>
@@ -11571,7 +11676,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -11595,6 +11700,11 @@
           <t>Hench LL. J Am Ceram Soc 1991;74:1487-1510 (vidros bioativos)</t>
         </is>
       </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+        </is>
+      </c>
       <c r="N172" t="n">
         <v>9</v>
       </c>
@@ -11632,7 +11742,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -11656,6 +11766,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+        </is>
+      </c>
       <c r="N173" t="n">
         <v>5</v>
       </c>
@@ -11693,7 +11808,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -11717,6 +11832,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+        </is>
+      </c>
       <c r="N174" t="n">
         <v>2</v>
       </c>
@@ -11754,7 +11874,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -11780,7 +11900,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N175" t="n">
@@ -11820,7 +11940,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -11846,7 +11966,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N176" t="n">
@@ -11886,7 +12006,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -11910,6 +12030,11 @@
           <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
         </is>
       </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+        </is>
+      </c>
       <c r="N177" t="n">
         <v>60</v>
       </c>
@@ -11947,7 +12072,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -11971,6 +12096,11 @@
           <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
         </is>
       </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+        </is>
+      </c>
       <c r="N178" t="n">
         <v>18</v>
       </c>
@@ -12008,7 +12138,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -12032,6 +12162,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+        </is>
+      </c>
       <c r="N179" t="n">
         <v>3</v>
       </c>
@@ -12069,7 +12204,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -12093,6 +12228,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+        </is>
+      </c>
       <c r="N180" t="n">
         <v>5</v>
       </c>
@@ -12130,7 +12270,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -12156,7 +12296,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N181" t="n">
@@ -12196,7 +12336,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -12222,7 +12362,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor</t>
+          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N182" t="n">
@@ -12262,7 +12402,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -12286,6 +12426,11 @@
           <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
         </is>
       </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte a indicar</t>
+        </is>
+      </c>
       <c r="N183" t="n">
         <v>87.5</v>
       </c>
@@ -12323,7 +12468,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -12347,6 +12492,11 @@
           <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
         </is>
       </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte a indicar</t>
+        </is>
+      </c>
       <c r="N184" t="n">
         <v>7.5</v>
       </c>
@@ -12384,7 +12534,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -12408,6 +12558,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte a indicar</t>
+        </is>
+      </c>
       <c r="N185" t="n">
         <v>3</v>
       </c>
@@ -12445,7 +12600,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -12469,6 +12624,11 @@
           <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
         </is>
       </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte a indicar</t>
+        </is>
+      </c>
       <c r="N186" t="n">
         <v>2</v>
       </c>
@@ -18169,7 +18329,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
@@ -18195,7 +18355,7 @@
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>Fusão ~60 °C: sem autoclave; EtO/gama com cuidado</t>
+          <t>Fusão ~60 °C: sem autoclave; EtO/gama com cuidado; Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
         </is>
       </c>
       <c r="N275" t="n">
@@ -18235,7 +18395,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
@@ -18261,7 +18421,7 @@
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>Gama causa cisão de cadeias</t>
+          <t>Gama causa cisão de cadeias; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N276" t="n">
@@ -18301,7 +18461,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -18327,7 +18487,7 @@
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>Muito sensível: altera a degradação</t>
+          <t>Muito sensível: altera a degradação; Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
         </is>
       </c>
       <c r="N277" t="n">
@@ -18367,7 +18527,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -18393,7 +18553,7 @@
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>Autoclave/calor seco</t>
+          <t>Autoclave/calor seco; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N278" t="n">
@@ -18433,7 +18593,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -18457,6 +18617,11 @@
           <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N279" t="n">
         <v>5</v>
       </c>
@@ -18494,7 +18659,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -18518,6 +18683,11 @@
           <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+        </is>
+      </c>
       <c r="N280" t="n">
         <v>5</v>
       </c>
@@ -18555,7 +18725,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
@@ -18581,7 +18751,7 @@
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>Limitado pela fase PCL</t>
+          <t>Limitado pela fase PCL; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N281" t="n">
@@ -18621,7 +18791,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
@@ -18647,7 +18817,7 @@
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>Polímero natural sensível ao calor</t>
+          <t>Polímero natural sensível ao calor; Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N282" t="n">
@@ -18687,7 +18857,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
@@ -18711,6 +18881,11 @@
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+        </is>
+      </c>
       <c r="N283" t="n">
         <v>1</v>
       </c>
@@ -18748,7 +18923,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
@@ -18772,6 +18947,11 @@
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+        </is>
+      </c>
       <c r="N284" t="n">
         <v>1</v>
       </c>
@@ -18809,7 +18989,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
@@ -18833,6 +19013,11 @@
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+        </is>
+      </c>
       <c r="N285" t="n">
         <v>2</v>
       </c>
@@ -18870,7 +19055,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
@@ -18894,6 +19079,11 @@
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N286" t="n">
         <v>3</v>
       </c>
@@ -18931,7 +19121,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -18955,6 +19145,11 @@
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
       <c r="N287" t="n">
         <v>3</v>
       </c>
@@ -18992,7 +19187,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -19016,6 +19211,11 @@
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+        </is>
+      </c>
       <c r="N288" t="n">
         <v>4</v>
       </c>
@@ -19053,7 +19253,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -19077,6 +19277,11 @@
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+        </is>
+      </c>
       <c r="N289" t="n">
         <v>2</v>
       </c>
@@ -19114,7 +19319,7 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>Clínico/investigação</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
@@ -19136,6 +19341,11 @@
       <c r="K290" t="inlineStr">
         <is>
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N290" t="n">

</xml_diff>

<commit_message>
Teor de níquel do stent com fontes, estados na legenda e nota da reunião de 28 set
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Parametros" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materiais'!$A$1:$P$290</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materiais'!$A$1:$P$296</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Criterios'!$A$1:$G$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Tecido'!$A$1:$H$9</definedName>
   </definedNames>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -609,154 +609,158 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>- Estados da coluna estado:</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
+          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
+          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
+          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
+          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>- Bioatividade: 5 = liga-se quimicamente ao osso; 4 = osteocondutor; 3 = compósito com fase bioativa; 1 = bioinerte</t>
-        </is>
-      </c>
+      <c r="A37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
+          <t>- Bioatividade: 5 = liga-se quimicamente ao osso; 4 = osteocondutor; 3 = compósito com fase bioativa; 1 = bioinerte</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Cuidados</t>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade: compara só valores com porosidades semelhantes, ou regista a porosidade.</t>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
-        </is>
-      </c>
+      <c r="A50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
         </is>
       </c>
     </row>
@@ -766,12 +770,50 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Níveis de validação</t>
+          <t>Cuidados</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
+        <is>
+          <t>1. Propriedades de scaffolds dependem da porosidade: compara só valores com porosidades semelhantes, ou regista a porosidade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Níveis de validação</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
         </is>
@@ -788,7 +830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P290"/>
+  <dimension ref="A1:P296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -802,10 +844,10 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="33" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
@@ -17933,12 +17975,12 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Co-Cr L605</t>
+          <t>Aço inox 316L</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>ASTM F90</t>
+          <t>ASTM F138</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -17948,36 +17990,46 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Clínico (1.ª geração)</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>Fabricabilidade (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I269" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="J269" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="K269" t="inlineStr">
         <is>
-          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
+          <t>Página de fornecedor (Upmet), 316L ASTM F138</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>https://www.upmet.com/products/stainless-steel/316lslvm</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>fonte: página de fornecedor que declara cumprir a norma, não o texto da norma ASTM</t>
         </is>
       </c>
       <c r="N269" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -17994,12 +18046,12 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Co-Ni-Cr-Mo MP35N</t>
+          <t>Co-Cr L605</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>ASTM F562</t>
+          <t>ASTM F90</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
@@ -18055,12 +18107,12 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Pt-Cr</t>
+          <t>Co-Cr L605</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F90</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -18075,31 +18127,41 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>Fabricabilidade (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I271" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J271" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
+          <t>Página de fornecedor (MGM Industries), L605 ASTM F90</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>https://www.mgm-industries.com/l605-alloy</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>fonte: página de fornecedor que declara cumprir a norma, não o texto da norma ASTM</t>
         </is>
       </c>
       <c r="N271" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -18116,22 +18178,22 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Nitinol (autoexpansível)</t>
+          <t>Co-Ni-Cr-Mo MP35N</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>ASTM F2063</t>
+          <t>ASTM F562</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Metal (superelástico)</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Excluído (autoexpansível: só discussão)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
@@ -18145,23 +18207,18 @@
         </is>
       </c>
       <c r="I272" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J272" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K272" t="inlineStr">
         <is>
           <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
-      <c r="M272" t="inlineStr">
-        <is>
-          <t>Tratamento de memória de forma</t>
-        </is>
-      </c>
       <c r="N272" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
@@ -18182,56 +18239,61 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Liga de Mg WE43 (bioabsorvível)</t>
+          <t>Co-Ni-Cr-Mo MP35N</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F562</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Metal biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Clínico (Magmaris)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>Fabricabilidade (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I273" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="J273" t="n">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
+          <t>Página de fornecedor (stainless.eu), MP35N ASTM F562</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>https://www.stainless.eu/en/products/cobalt-alloys/mp35n/</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>Controlo de degradação e revestimentos</t>
+          <t>fonte: página de fornecedor que declara cumprir a norma, não o texto da norma ASTM</t>
         </is>
       </c>
       <c r="N273" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -18248,7 +18310,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>PLLA (bioabsorvível)</t>
+          <t>Pt-Cr</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -18258,12 +18320,12 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Polímero biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>Descontinuado (Absorb, 2017)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -18277,23 +18339,18 @@
         </is>
       </c>
       <c r="I274" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J274" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K274" t="inlineStr">
         <is>
           <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
-      <c r="M274" t="inlineStr">
-        <is>
-          <t>Struts espessos; processamento térmico sensível</t>
-        </is>
-      </c>
       <c r="N274" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
@@ -18304,17 +18361,17 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>PCL</t>
+          <t>Pt-Cr</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -18324,83 +18381,88 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>Clínico (uso limitado)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I275" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J275" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>A novel platinum chromium everolimus-eluting stent for the treatment of coronary artery disease. Biologics: Targets and Therapy 2013;7:149 [confirmar autores e ano]</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2147/BTT.S34939</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
         <is>
-          <t>Fusão ~60 °C: sem autoclave; EtO/gama com cuidado; Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+          <t>valor nominal, sem intervalo (PMC3692344: 33 % Fe, 33 % Pt, 18 % Cr, 9 % Ni, 3 % Mo)</t>
         </is>
       </c>
       <c r="N275" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>PLLA</t>
+          <t>Nitinol (autoexpansível)</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F2063</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Metal (superelástico)</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Investigação</t>
+          <t>Excluído (autoexpansível: só discussão)</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Fabricabilidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -18416,12 +18478,12 @@
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>Gama causa cisão de cadeias; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+          <t>Tratamento de memória de forma</t>
         </is>
       </c>
       <c r="N276" t="n">
@@ -18436,17 +18498,17 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>PLGA 50:50</t>
+          <t>Liga de Mg WE43 (bioabsorvível)</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -18456,17 +18518,17 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Metal biodegradável</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Investigação</t>
+          <t>Clínico (Magmaris)</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Fabricabilidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
@@ -18475,23 +18537,23 @@
         </is>
       </c>
       <c r="I277" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J277" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
       <c r="M277" t="inlineStr">
         <is>
-          <t>Muito sensível: altera a degradação; Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+          <t>Controlo de degradação e revestimentos</t>
         </is>
       </c>
       <c r="N277" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -18502,17 +18564,17 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Hidroxiapatite (HA) porosa</t>
+          <t>Liga de Mg WE43 (bioabsorvível)</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -18522,42 +18584,47 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Cerâmico</t>
+          <t>Metal biodegradável</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo)</t>
+          <t>Clínico (Magmaris)</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I278" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J278" t="n">
-        <v>5</v>
+        <v>0.005</v>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>MakeItFrom, WE43B (cita ASTM B80)</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>https://www.makeitfrom.com/material-properties/WE43B-WE43B-T6-M18432-Magnesium</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>Autoclave/calor seco; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>limite máximo de Ni como impureza; típico = máximo (pior caso); fonte secundária; a ficha Luxfer DS-467 (05/2026) não indica Ni; composição da liga do Magmaris não confirmada</t>
         </is>
       </c>
       <c r="N278" t="n">
-        <v>5</v>
+        <v>0.005</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
@@ -18568,17 +18635,17 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>β-TCP poroso</t>
+          <t>PLLA (bioabsorvível)</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -18588,17 +18655,17 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Cerâmico</t>
+          <t>Polímero biodegradável</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo)</t>
+          <t>Descontinuado (Absorb, 2017)</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Fabricabilidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H279" t="inlineStr">
@@ -18607,23 +18674,23 @@
         </is>
       </c>
       <c r="I279" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J279" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>Struts espessos; processamento térmico sensível</t>
         </is>
       </c>
       <c r="N279" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -18634,17 +18701,17 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Vidro bioativo 45S5 poroso</t>
+          <t>PLLA (bioabsorvível)</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -18654,46 +18721,46 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Vidro</t>
+          <t>Polímero biodegradável</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo, partículas)</t>
+          <t>Descontinuado (Absorb, 2017)</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I280" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J280" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Composição química do PLLA</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+          <t>polímero de C, H e O; sem metais</t>
         </is>
       </c>
       <c r="N280" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (composição química)</t>
         </is>
       </c>
     </row>
@@ -18710,7 +18777,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Compósito PCL/β-TCP (impressão 3D)</t>
+          <t>PCL</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -18720,7 +18787,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Compósito</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
@@ -18751,7 +18818,7 @@
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>Limitado pela fase PCL; Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>Fusão ~60 °C: sem autoclave; EtO/gama com cuidado; Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
         </is>
       </c>
       <c r="N281" t="n">
@@ -18776,7 +18843,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Quitosano/HA (liofilizado)</t>
+          <t>PLLA</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -18786,7 +18853,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Compósito natural</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -18817,7 +18884,7 @@
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>Polímero natural sensível ao calor; Estatuto [confirmar]: fonte a indicar</t>
+          <t>Gama causa cisão de cadeias; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N282" t="n">
@@ -18842,7 +18909,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>PCL</t>
+          <t>PLGA 50:50</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -18857,12 +18924,12 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Clínico (uso limitado)</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
@@ -18871,23 +18938,23 @@
         </is>
       </c>
       <c r="I283" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J283" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+          <t>Muito sensível: altera a degradação; Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
         </is>
       </c>
       <c r="N283" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
@@ -18908,7 +18975,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>PLLA</t>
+          <t>Hidroxiapatite (HA) porosa</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -18918,17 +18985,17 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Cerâmico</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>Investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
@@ -18937,23 +19004,23 @@
         </is>
       </c>
       <c r="I284" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J284" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+          <t>Autoclave/calor seco; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N284" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -18974,7 +19041,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>PLGA 50:50</t>
+          <t>β-TCP poroso</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -18984,17 +19051,17 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Cerâmico</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
@@ -19003,23 +19070,23 @@
         </is>
       </c>
       <c r="I285" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J285" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N285" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
@@ -19040,7 +19107,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Hidroxiapatite (HA) porosa</t>
+          <t>Vidro bioativo 45S5 poroso</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -19050,17 +19117,17 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Cerâmico</t>
+          <t>Vidro</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo)</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H286" t="inlineStr">
@@ -19069,23 +19136,23 @@
         </is>
       </c>
       <c r="I286" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J286" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K286" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
         </is>
       </c>
       <c r="N286" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -19106,7 +19173,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>β-TCP poroso</t>
+          <t>Compósito PCL/β-TCP (impressão 3D)</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -19116,17 +19183,17 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Cerâmico</t>
+          <t>Compósito</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo)</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
@@ -19142,12 +19209,12 @@
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>Limitado pela fase PCL; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N287" t="n">
@@ -19172,7 +19239,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Vidro bioativo 45S5 poroso</t>
+          <t>Quitosano/HA (liofilizado)</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -19182,17 +19249,17 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Vidro</t>
+          <t>Compósito natural</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo, partículas)</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
@@ -19201,23 +19268,23 @@
         </is>
       </c>
       <c r="I288" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J288" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M288" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+          <t>Polímero natural sensível ao calor; Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N288" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
@@ -19238,7 +19305,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Compósito PCL/β-TCP (impressão 3D)</t>
+          <t>PCL</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -19248,7 +19315,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Compósito</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -19267,10 +19334,10 @@
         </is>
       </c>
       <c r="I289" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J289" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K289" t="inlineStr">
         <is>
@@ -19279,11 +19346,11 @@
       </c>
       <c r="M289" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
         </is>
       </c>
       <c r="N289" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O289" t="inlineStr">
         <is>
@@ -19304,61 +19371,457 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
+          <t>PLLA</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Polímero</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Investigação</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>1</v>
+      </c>
+      <c r="J290" t="n">
+        <v>1</v>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+        </is>
+      </c>
+      <c r="N290" t="n">
+        <v>1</v>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>PLGA 50:50</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Polímero</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Investigação</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>2</v>
+      </c>
+      <c r="J291" t="n">
+        <v>2</v>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+        </is>
+      </c>
+      <c r="N291" t="n">
+        <v>2</v>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Hidroxiapatite (HA) porosa</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Cerâmico</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Clínico (substituto ósseo)</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>3</v>
+      </c>
+      <c r="J292" t="n">
+        <v>3</v>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
+      <c r="N292" t="n">
+        <v>3</v>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>β-TCP poroso</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Cerâmico</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Clínico (substituto ósseo)</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>3</v>
+      </c>
+      <c r="J293" t="n">
+        <v>3</v>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
+      <c r="N293" t="n">
+        <v>3</v>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Vidro bioativo 45S5 poroso</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Vidro</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Clínico (substituto ósseo, partículas)</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>4</v>
+      </c>
+      <c r="J294" t="n">
+        <v>4</v>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+        </is>
+      </c>
+      <c r="N294" t="n">
+        <v>4</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Compósito PCL/β-TCP (impressão 3D)</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Compósito</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Clínico (uso limitado)</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>2</v>
+      </c>
+      <c r="J295" t="n">
+        <v>2</v>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+        </is>
+      </c>
+      <c r="N295" t="n">
+        <v>2</v>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
           <t>Quitosano/HA (liofilizado)</t>
         </is>
       </c>
-      <c r="D290" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E290" t="inlineStr">
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
         <is>
           <t>Compósito natural</t>
         </is>
       </c>
-      <c r="F290" t="inlineStr">
+      <c r="F296" t="inlineStr">
         <is>
           <t>Investigação</t>
         </is>
       </c>
-      <c r="G290" t="inlineStr">
+      <c r="G296" t="inlineStr">
         <is>
           <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
         </is>
       </c>
-      <c r="H290" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I290" t="n">
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
         <v>2</v>
       </c>
-      <c r="J290" t="n">
+      <c r="J296" t="n">
         <v>2</v>
       </c>
-      <c r="K290" t="inlineStr">
+      <c r="K296" t="inlineStr">
         <is>
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
-      <c r="M290" t="inlineStr">
+      <c r="M296" t="inlineStr">
         <is>
           <t>Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
-      <c r="N290" t="n">
+      <c r="N296" t="n">
         <v>2</v>
       </c>
-      <c r="O290" t="inlineStr">
+      <c r="O296" t="inlineStr">
         <is>
           <t>A verificar</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P290"/>
+  <autoFilter ref="A1:P296"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Correções da haste com fontes verificadas (Li 2014, Navarro 2008, Okazaki 2012), resultados atualizados e tabela do par articular
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A60"/>
+  <dimension ref="A1:A61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -646,174 +646,181 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
-        </is>
-      </c>
+      <c r="A35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-    </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
-        </is>
-      </c>
+      <c r="A38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
+          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>- Bioatividade: 5 = liga-se quimicamente ao osso; 4 = osteocondutor; 3 = compósito com fase bioativa; 1 = bioinerte</t>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+          <t>- Bioatividade: 5 = liga-se quimicamente ao osso; 4 = osteocondutor; 3 = compósito com fase bioativa; 1 = bioinerte</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-    </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-    </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Cuidados</t>
-        </is>
-      </c>
+      <c r="A53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade: compara só valores com porosidades semelhantes, ou regista a porosidade.</t>
+          <t>Cuidados</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+          <t>1. Propriedades de scaffolds dependem da porosidade: compara só valores com porosidades semelhantes, ou regista a porosidade.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr"/>
-    </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Níveis de validação</t>
-        </is>
-      </c>
+      <c r="A59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
+        <is>
+          <t>Níveis de validação</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
         </is>
@@ -975,27 +982,32 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="J2" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Navarro M, Michiardi A, Castaño O, Planell JA. Biomaterials in orthopaedics. J R Soc Interface 2008;5(27):1137-1158</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1098/rsif.2008.0151</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Valores dependem muito de recozido vs encruado</t>
+          <t>Navarro et al. 2008, Tabela 1: 205-210 GPa; típico = ponto médio</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>195</v>
+        <v>207.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -1041,27 +1053,32 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>190</v>
+        <v>755</v>
       </c>
       <c r="J3" t="n">
-        <v>690</v>
+        <v>765</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Okazaki Y. Comparison of Fatigue Properties and Fatigue Crack Growth Rates of Various Implantable Metals. Materials 2012;5:2981</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma5122981</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Valores dependem muito de recozido vs encruado</t>
+          <t>hastes em 316L usam aço encruado; o recozido fica fora por fadiga insuficiente [fonte a indicar]; aço ISO 5832-1, 20 % encruado; Okazaki 2012, Tabela 2: σ0,2 = 760 ± 5 MPa (mín.-máx. = média ± DP)</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>440</v>
+        <v>760</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -1173,27 +1190,32 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>180</v>
+        <v>694</v>
       </c>
       <c r="J5" t="n">
-        <v>380</v>
+        <v>694</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Okazaki Y. Comparison of Fatigue Properties and Fatigue Crack Growth Rates of Various Implantable Metals. Materials 2012;5:2981</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma5122981</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Valores dependem muito de recozido vs encruado</t>
+          <t>hastes em 316L usam aço encruado; o recozido fica fora por fadiga insuficiente [fonte a indicar]; aço ISO 5832-1, 20 % encruado; Okazaki 2012, Tabela 2: σFS/σUTS = 0,79 e σUTS = 878 ± 19 MPa; cálculo: 0,79 × 878 = 694 MPa; ensaio tração-tração, R = 0,1, 10 Hz, meio de Eagle a 37 °C</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>280</v>
+        <v>694</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (derivado)</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1268,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>[fonte a indicar] (o Niinomi 1998 é só de ligas de Ti)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1371,19 +1393,24 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="J8" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Navarro M, Michiardi A, Castaño O, Planell JA. Biomaterials in orthopaedics. J R Soc Interface 2008;5(27):1137-1158</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1098/rsif.2008.0151</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Slides: F799 ~2x fadiga/cedência da F75</t>
+          <t>Navarro et al. 2008, Tabela 1 (linha CoCrMo F75): 220-230 GPa; típico = ponto médio; o módulo quase não depende do processamento (fundido ou forjado)</t>
         </is>
       </c>
       <c r="N8" t="n">
@@ -1391,7 +1418,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -1437,27 +1464,32 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>700</v>
+        <v>629</v>
       </c>
       <c r="J9" t="n">
-        <v>1000</v>
+        <v>709</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Okazaki Y. Comparison of Fatigue Properties and Fatigue Crack Growth Rates of Various Implantable Metals. Materials 2012;5:2981</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma5122981</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Slides: F799 ~2x fadiga/cedência da F75</t>
+          <t>Forjado a quente; Okazaki 2012, Tabela 2: σ0,2 = 669 ± 40 MPa (mín.-máx. = média ± DP)</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>850</v>
+        <v>669</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -1569,27 +1601,32 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>600</v>
+        <v>796</v>
       </c>
       <c r="J11" t="n">
-        <v>900</v>
+        <v>796</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Okazaki Y. Comparison of Fatigue Properties and Fatigue Crack Growth Rates of Various Implantable Metals. Materials 2012;5:2981</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma5122981</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Slides: F799 ~2x fadiga/cedência da F75</t>
+          <t>Forjado a quente; Okazaki 2012, Tabela 2: σFS/σUTS = 0,74 e σUTS = 1075 ± 20 MPa; cálculo: 0,74 × 1075 = 796 MPa; ensaio tração-tração, R = 0,1, 10 Hz, meio de Eagle a 37 °C</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>750</v>
+        <v>796</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (derivado)</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1679,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>[fonte a indicar] (o Niinomi 1998 é só de ligas de Ti)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1767,22 +1804,32 @@
         </is>
       </c>
       <c r="I14" t="n">
+        <v>101</v>
+      </c>
+      <c r="J14" t="n">
         <v>110</v>
       </c>
-      <c r="J14" t="n">
-        <v>114</v>
-      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Li et al. 2014, Tabela 4 (cita Niinomi 1998): 101-110 GPa, recozido; típico = ponto médio; o valor 110-114 anterior era do Ti-6Al-4V normal (ASTM F1472), não do ELI</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>112</v>
+        <v>105.5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1882,17 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Li et al. 2014, Tabela 4 (cita Niinomi 1998): 795-875 MPa, recozido; típico = ponto médio</t>
         </is>
       </c>
       <c r="N15" t="n">
@@ -1843,7 +1900,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -2133,27 +2190,32 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>103</v>
+        <v>104.1</v>
       </c>
       <c r="J20" t="n">
-        <v>110</v>
+        <v>104.1</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Resistência limitada para haste de carga elevada</t>
+          <t>Resistência limitada para haste de carga elevada; Li et al. 2014, Tabela 4 (cita Niinomi 1998): 104,1 GPa, recozido; a ASTM F67 não especifica módulo: mín. = máx. = típico</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>106.5</v>
+        <v>104.1</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -2199,27 +2261,32 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="J21" t="n">
-        <v>550</v>
+        <v>485</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Resistência limitada para haste de carga elevada</t>
+          <t>Resistência limitada para haste de carga elevada; típico = Li et al. 2014, Tabela 4 (cita Niinomi 1998): 485 MPa, recozido (o 550 anterior era a tensão de rotura); mín. = mínimo da ASTM F67 grau 4 recozido (483 MPa), segundo página de fornecedor (gsalloy.com), não o texto da norma; a norma não tem máximo, máx. = típico</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>515</v>
+        <v>485</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -2536,12 +2603,17 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Geetha M et al. Prog Mater Sci 2009;54:397-425</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Liga β sem Al/V, módulo mais baixo</t>
+          <t>Liga β sem Al/V, módulo mais baixo; Li et al. 2014, Tabela 4 (cita Niinomi 1998): 79-84 GPa, envelhecido; típico = ponto médio</t>
         </is>
       </c>
       <c r="N26" t="n">
@@ -2549,7 +2621,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -2602,12 +2674,17 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Geetha M et al. Prog Mater Sci 2009;54:397-425</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Liga β sem Al/V, módulo mais baixo</t>
+          <t>Liga β sem Al/V, módulo mais baixo; Li et al. 2014, Tabela 4 (cita Niinomi 1998): 836-908 MPa, envelhecido; típico = ponto médio</t>
         </is>
       </c>
       <c r="N27" t="n">
@@ -2615,7 +2692,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -2928,24 +3005,29 @@
         <v>55</v>
       </c>
       <c r="J32" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Geetha M et al. Prog Mater Sci 2009;54:397-425</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Excluído no cenário 'só materiais clínicos'</t>
+          <t>Excluído no cenário 'só materiais clínicos'; variante com 0,06 % de O; Li et al. 2014, Tabela 4 (recozido): 55 GPa; o valor de 66 GPa corresponde à variante com mais oxigénio (0,4 % O)</t>
         </is>
       </c>
       <c r="N32" t="n">
-        <v>60.5</v>
+        <v>55</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -2994,24 +3076,29 @@
         <v>530</v>
       </c>
       <c r="J33" t="n">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Geetha M et al. Prog Mater Sci 2009;54:397-425</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Excluído no cenário 'só materiais clínicos'</t>
+          <t>Excluído no cenário 'só materiais clínicos'; variante com 0,06 % de O; Li et al. 2014: 530 MPa (Tabela 11, 0,06 % O, solubilizado) e 547 MPa (Tabela 4, recozido); típico = ponto médio</t>
         </is>
       </c>
       <c r="N33" t="n">
-        <v>540</v>
+        <v>538.5</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -3123,27 +3210,32 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="J35" t="n">
-        <v>450</v>
+        <v>275</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Geetha M et al. Prog Mater Sci 2009;54:397-425</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Excluído no cenário 'só materiais clínicos'</t>
+          <t>Excluído no cenário 'só materiais clínicos'; variante com 0,06 % de O; Li et al. 2014, secção 4.1 (texto): 275 MPa, solubilizado; o valor de 450 MPa corresponde à variante com mais oxigénio (0,46 % O)</t>
         </is>
       </c>
       <c r="N35" t="n">
-        <v>357.5</v>
+        <v>275</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -21592,19 +21684,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="D2" t="n">
-        <v>9.5</v>
+        <v>10.25</v>
       </c>
       <c r="E2" t="n">
-        <v>11.143</v>
+        <v>11.857</v>
       </c>
       <c r="F2" t="n">
-        <v>13.333</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -21614,19 +21706,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="C3" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="D3" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="E3" t="n">
         <v>12.857</v>
       </c>
       <c r="F3" t="n">
-        <v>16</v>
+        <v>15.333</v>
       </c>
     </row>
     <row r="4">
@@ -21636,19 +21728,19 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>101</v>
+      </c>
+      <c r="C4" t="n">
         <v>110</v>
       </c>
-      <c r="C4" t="n">
-        <v>114</v>
-      </c>
       <c r="D4" t="n">
-        <v>5.5</v>
+        <v>5.05</v>
       </c>
       <c r="E4" t="n">
-        <v>6.4</v>
+        <v>6.029</v>
       </c>
       <c r="F4" t="n">
-        <v>7.6</v>
+        <v>7.333</v>
       </c>
     </row>
     <row r="5">
@@ -21658,19 +21750,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>103</v>
+        <v>104.1</v>
       </c>
       <c r="C5" t="n">
-        <v>110</v>
+        <v>104.1</v>
       </c>
       <c r="D5" t="n">
-        <v>5.15</v>
+        <v>5.205</v>
       </c>
       <c r="E5" t="n">
-        <v>6.086</v>
+        <v>5.949</v>
       </c>
       <c r="F5" t="n">
-        <v>7.333</v>
+        <v>6.94</v>
       </c>
     </row>
     <row r="6">
@@ -21705,16 +21797,16 @@
         <v>55</v>
       </c>
       <c r="C7" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="D7" t="n">
         <v>2.75</v>
       </c>
       <c r="E7" t="n">
-        <v>3.457</v>
+        <v>3.143</v>
       </c>
       <c r="F7" t="n">
-        <v>4.4</v>
+        <v>3.667</v>
       </c>
     </row>
   </sheetData>
@@ -21976,7 +22068,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
@@ -22047,17 +22139,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Longitudinal; anisotrópico (slide 10)</t>
+          <t>Longitudinal; anisotrópico (slide 10); Li et al. 2014, Tabelas 1 e 2 (fémur): 13,6-16,8 GPa em tração, 17,6 GPa em compressão; osso de idosos pode ficar abaixo de 15 GPa: relevante para o perfil osteoporose</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ratner et al. 2020; Navarro et al. 2008; Karageorgiou &amp; Kaplan 2005: confirmar</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications), Tabelas 1 e 2, https://doi.org/10.3390/ma7031709; Ratner et al. 2020; Navarro et al. 2008; Karageorgiou &amp; Kaplan 2005: confirmar</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fadiga e cedência do Ti-6Al-4V e do Ti cp grau 4 pelo Okazaki 2012 e limitações nas notas
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -1875,28 +1875,28 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>795</v>
+        <v>848</v>
       </c>
       <c r="J15" t="n">
-        <v>875</v>
+        <v>850</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+          <t>Okazaki Y. Comparison of Fatigue Properties and Fatigue Crack Growth Rates of Various Implantable Metals. Materials 2012;5:2981</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/ma7031709</t>
+          <t>https://doi.org/10.3390/ma5122981</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Li et al. 2014, Tabela 4 (cita Niinomi 1998): 795-875 MPa, recozido; típico = ponto médio</t>
+          <t>Okazaki 2012, Ti-6Al-4V ISO 5832-3 recozido; o artigo não diz se é ELI (O medido 0,07 %); Tabela 2: σ0,2 = 849 ± 1 MPa (mín.-máx. = média ± DP); valor anterior: 795-875 MPa (Li et al. 2014, Tabela 4, ELI recozido)</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>835</v>
+        <v>849</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -2007,22 +2007,32 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>500</v>
+        <v>682</v>
       </c>
       <c r="J17" t="n">
-        <v>650</v>
+        <v>682</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Okazaki Y. Comparison of Fatigue Properties and Fatigue Crack Growth Rates of Various Implantable Metals. Materials 2012;5:2981</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma5122981</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Okazaki 2012, Ti-6Al-4V ISO 5832-3 recozido; o artigo não diz se é ELI (O medido 0,07 %); Tabela 2: σFS/σUTS = 0,73 e σUTS = 934 ± 1 MPa; cálculo: 0,73 × 934 = 682 MPa; ensaio tração-tração, R = 0,1, 10 Hz, ao ar (Figura 7); valor anterior: 500-650 MPa (Niinomi 1998, A verificar)</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>575</v>
+        <v>682</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (derivado)</t>
         </is>
       </c>
     </row>
@@ -2261,28 +2271,28 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>483</v>
+        <v>610</v>
       </c>
       <c r="J21" t="n">
-        <v>485</v>
+        <v>622</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+          <t>Okazaki Y. Comparison of Fatigue Properties and Fatigue Crack Growth Rates of Various Implantable Metals. Materials 2012;5:2981</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://doi.org/10.3390/ma7031709</t>
+          <t>https://doi.org/10.3390/ma5122981</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Resistência limitada para haste de carga elevada; típico = Li et al. 2014, Tabela 4 (cita Niinomi 1998): 485 MPa, recozido (o 550 anterior era a tensão de rotura); mín. = mínimo da ASTM F67 grau 4 recozido (483 MPa), segundo página de fornecedor (gsalloy.com), não o texto da norma; a norma não tem máximo, máx. = típico</t>
+          <t>Resistência limitada para haste de carga elevada; Okazaki 2012, Ti cp grau 4 (ISO 5832-2) recozido; Tabela 2: σ0,2 = 616 ± 6 MPa (mín.-máx. = média ± DP); valor anterior: 483-485 MPa (Li et al. 2014, Tabela 4: 485 MPa; mínimo da ASTM F67: 483 MPa)</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>485</v>
+        <v>616</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2398,27 +2408,32 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>340</v>
+        <v>483</v>
       </c>
       <c r="J23" t="n">
-        <v>430</v>
+        <v>483</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Okazaki Y. Comparison of Fatigue Properties and Fatigue Crack Growth Rates of Various Implantable Metals. Materials 2012;5:2981</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma5122981</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Resistência limitada para haste de carga elevada</t>
+          <t>Resistência limitada para haste de carga elevada; Okazaki 2012, Ti cp grau 4 (ISO 5832-2) recozido; Tabela 2: σFS/σUTS = 0,69 e σUTS = 700 ± 8 MPa; cálculo: 0,69 × 700 = 483 MPa; ensaio tração-tração, R = 0,1, 10 Hz, meio não indicado; valor anterior: 340-430 MPa (Niinomi 1998, A verificar)</t>
         </is>
       </c>
       <c r="N23" t="n">
-        <v>385</v>
+        <v>483</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (derivado)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Par articular: desgaste in vivo e dureza da cabeça com fontes verificadas, simulador à parte na tabela de apoio
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -3428,27 +3428,32 @@
         </is>
       </c>
       <c r="I38" t="n">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="J38" t="n">
-        <v>0.2</v>
+        <v>0.106</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Kurtz SM. UHMWPE Biomaterials Handbook, 3rd ed., 2016</t>
+          <t>Teeter MG, Yuan X, Somerville LE, MacDonald SJ, McCalden RW, Naudie DD. Thirteen-year wear rate comparison of highly crosslinked and conventional polyethylene in total hip arthroplasty. Can J Surg 2017;60(3):212-216</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1503/cjs.005216</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | Osteólise por partículas de PE; corrosão na junção cabeça-cone</t>
+          <t>in vivo, RSA; CoCr 28 mm contra PE convencional (Trilogy, Zimmer); ensaio aleatorizado, n = 8 por braço aos 13,6 anos; rodagem incluída; mín.-máx. = intervalo; sem rodagem (primeiros 5 anos): 0,051 ± 0,022 mm/ano; Glyn-Jones 2015 (RSA): 0,030 mm/ano em regime estacionário, cabeça não indicada; mistura de métodos: RSA neste par, radiografia simples nos restantes | Osteólise por partículas de PE; corrosão na junção cabeça-cone</t>
         </is>
       </c>
       <c r="N38" t="n">
-        <v>0.15</v>
+        <v>0.077</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -3494,27 +3499,32 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="J39" t="n">
-        <v>450</v>
+        <v>368</v>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Chevalier J. Biomaterials 2006;27:535-543 (zircónia/envelhecimento)</t>
+          <t>Fischer A, Weiß S, Wimmer MA. The tribological difference between biomedical steels and CoCrMo-alloys. J Mech Behav Biomed Mater 2012;9:50-62, Tabela 1</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jmbbm.2012.01.007</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | Osteólise por partículas de PE; corrosão na junção cabeça-cone</t>
+          <t>varão forjado, não cabeça femoral; HV10 = 340 ± 28 (mín.-máx. = média ± DP); CoCr29Mo6 de baixo carbono, ISO 5832-6 / ASTM F1537, solubilizado | Osteólise por partículas de PE; corrosão na junção cabeça-cone</t>
         </is>
       </c>
       <c r="N39" t="n">
-        <v>375</v>
+        <v>340</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -3626,27 +3636,32 @@
         </is>
       </c>
       <c r="I41" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
       <c r="J41" t="n">
-        <v>0.05</v>
+        <v>0.0212</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Kurtz SM. UHMWPE Biomaterials Handbook, 3rd ed., 2016</t>
+          <t>Higuchi Y, Seki T, Morita D, Komatsu D, Takegami Y, Ishiguro N. Comparison of wear rate between ceramic-on-ceramic, metal on highly cross-linked polyethylene, and metal-on-metal bearings. Rev Bras Ortop 2019;54(3):295-302, Tabela 4</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1055/s-0039-1691762</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | PE altamente reticulado; oxidação se radiação gama sem estabilização</t>
+          <t>in vivo, radiografia simples (AP); CoCr contra HXLPE Crossfire (Stryker); n = 77; 7,6 anos; média ± DP; rodagem incluída; sem rodagem (true wear): 0,0096 mm/ano | PE altamente reticulado; oxidação se radiação gama sem estabilização</t>
         </is>
       </c>
       <c r="N41" t="n">
-        <v>0.03</v>
+        <v>0.0161</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -3692,27 +3707,32 @@
         </is>
       </c>
       <c r="I42" t="n">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="J42" t="n">
-        <v>450</v>
+        <v>368</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Chevalier J. Biomaterials 2006;27:535-543 (zircónia/envelhecimento)</t>
+          <t>Fischer A, Weiß S, Wimmer MA. The tribological difference between biomedical steels and CoCrMo-alloys. J Mech Behav Biomed Mater 2012;9:50-62, Tabela 1</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jmbbm.2012.01.007</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | PE altamente reticulado; oxidação se radiação gama sem estabilização</t>
+          <t>varão forjado, não cabeça femoral; HV10 = 340 ± 28 (mín.-máx. = média ± DP); CoCr29Mo6 de baixo carbono, ISO 5832-6 / ASTM F1537, solubilizado | PE altamente reticulado; oxidação se radiação gama sem estabilização</t>
         </is>
       </c>
       <c r="N42" t="n">
-        <v>375</v>
+        <v>340</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -3824,27 +3844,32 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>0.01</v>
+        <v>0.032</v>
       </c>
       <c r="J44" t="n">
-        <v>0.04</v>
+        <v>0.044</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Kurtz SM. UHMWPE Biomaterials Handbook, 3rd ed., 2016</t>
+          <t>Kim YH, Park JW. Eighteen-Year Results of Cementless THA with Alumina-on-HXLPE Bearings in Patients &lt;30 Years Old. J Bone Joint Surg Am 2020;102(14):1255-1259</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2106/JBJS.19.01157</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | Cerâmica na cabeça elimina corrosão na junção</t>
+          <t>alumina BIOLOX forte, não ZTA; doentes &lt; 30 anos (muito ativos): pior caso; não comparável com o MoXLPE, porque os estudos, os polietilenos e os métodos são diferentes; in vivo, radiografia simples (AP, AutoCAD); 28 mm contra HXLPE Marathon (DePuy); cerca de 54 ancas; 17,8 anos; média ± DP; tratamento da rodagem não explicado; Weishorn 2023: 0,059 ± 0,031 mm/ano sem rodagem (Biolox sem geração indicada, contra Durasul); Dahl 2013 (RSA, PE convencional): a cabeça de alumina desgastou o PE menos de metade da CoCr (0,62 vs 1,40 mm aos 10 anos), única comparação cerâmica vs CoCr no mesmo estudo | Cerâmica na cabeça elimina corrosão na junção</t>
         </is>
       </c>
       <c r="N44" t="n">
-        <v>0.025</v>
+        <v>0.038</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -3890,27 +3915,32 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>1750</v>
+        <v>1937</v>
       </c>
       <c r="J45" t="n">
-        <v>1975</v>
+        <v>1937</v>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Chevalier J. Biomaterials 2006;27:535-543 (zircónia/envelhecimento)</t>
+          <t>KYOCERA Medical Technologies. BIOLOX delta Ceramic (página de produto), Tabela 1; consultada a 29 set 2026</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>https://medical.kyocera.com/joint/prdct/biolox-delta-ceramic.html</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | Cerâmica na cabeça elimina corrosão na junção</t>
+          <t>BIOLOX delta; fonte: página de distribuidor (Kyocera), não o fabricante: 19 GPa (HV1); conversão: 19 / 0,009807 = 1937 HV; apoio: Merkert 2008 (resumo de congresso): 1975 HV; DePuy (folheto): cerca de 2000 HV | Cerâmica na cabeça elimina corrosão na junção</t>
         </is>
       </c>
       <c r="N45" t="n">
-        <v>1862.5</v>
+        <v>1937</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -4022,27 +4052,32 @@
         </is>
       </c>
       <c r="I47" t="n">
-        <v>0.001</v>
+        <v>0.0019</v>
       </c>
       <c r="J47" t="n">
-        <v>0.005</v>
+        <v>0.0063</v>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Kurtz SM. UHMWPE Biomaterials Handbook, 3rd ed., 2016</t>
+          <t>Higuchi Y, Seki T, Morita D, Komatsu D, Takegami Y, Ishiguro N. Comparison of wear rate between ceramic-on-ceramic, metal on highly cross-linked polyethylene, and metal-on-metal bearings. Rev Bras Ortop 2019;54(3):295-302, Tabela 4</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1055/s-0039-1691762</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | Risco de fratura baixo mas não nulo; ruído (squeaking)</t>
+          <t>alumina, não ZTA; a ZTA desgasta igual ou menos, logo é o pior caso; in vivo, radiografia simples (AP); BIOLOX forte; n = 105; 7,6 anos; média ± DP; rodagem incluída (sem rodagem: 0,0037 mm/ano); van Loon 2021 (BIOLOX delta, 32 mm, n = 25 aos 10 anos): mediana 0,000 mm/ano (0,000 a 0,005); valores abaixo da resolução da radiografia simples: a diferença entre CoC e MoM não é significativa | Risco de fratura baixo mas não nulo; ruído (squeaking)</t>
         </is>
       </c>
       <c r="N47" t="n">
-        <v>0.003</v>
+        <v>0.0041</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -4088,27 +4123,32 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>1750</v>
+        <v>1937</v>
       </c>
       <c r="J48" t="n">
-        <v>1975</v>
+        <v>1937</v>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Chevalier J. Biomaterials 2006;27:535-543 (zircónia/envelhecimento)</t>
+          <t>KYOCERA Medical Technologies. BIOLOX delta Ceramic (página de produto), Tabela 1; consultada a 29 set 2026</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>https://medical.kyocera.com/joint/prdct/biolox-delta-ceramic.html</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | Risco de fratura baixo mas não nulo; ruído (squeaking)</t>
+          <t>BIOLOX delta; fonte: página de distribuidor (Kyocera), não o fabricante: 19 GPa (HV1); conversão: 19 / 0,009807 = 1937 HV; apoio: Merkert 2008 (resumo de congresso): 1975 HV; DePuy (folheto): cerca de 2000 HV | Risco de fratura baixo mas não nulo; ruído (squeaking)</t>
         </is>
       </c>
       <c r="N48" t="n">
-        <v>1862.5</v>
+        <v>1937</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -4220,27 +4260,32 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>0.003</v>
+        <v>0.0035</v>
       </c>
       <c r="J50" t="n">
-        <v>0.01</v>
+        <v>0.0073</v>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Kurtz SM. UHMWPE Biomaterials Handbook, 3rd ed., 2016</t>
+          <t>Higuchi Y, Seki T, Morita D, Komatsu D, Takegami Y, Ishiguro N. Comparison of wear rate between ceramic-on-ceramic, metal on highly cross-linked polyethylene, and metal-on-metal bearings. Rev Bras Ortop 2019;54(3):295-302, Tabela 4</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1055/s-0039-1691762</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | Iões Co/Cr, ALTR; recolha ASR 2010: candidato a eliminar na triagem</t>
+          <t>in vivo, radiografia simples (AP); Pinnacle 28 e 36 mm; n = 55; 7,6 anos; média ± DP; rodagem incluída (sem rodagem: 0,0051 mm/ano); Sieber 1999 (explantes Metasul, n = 118): cerca de 25 µm/ano no 1.º ano e 5 µm/ano depois do 3.º [confirmar: só o resumo]; valores abaixo da resolução da radiografia simples: a diferença entre CoC e MoM não é significativa | Iões Co/Cr, ALTR; recolha ASR 2010: candidato a eliminar na triagem</t>
         </is>
       </c>
       <c r="N50" t="n">
-        <v>0.0065</v>
+        <v>0.0054</v>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -4286,27 +4331,32 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="J51" t="n">
-        <v>450</v>
+        <v>368</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Chevalier J. Biomaterials 2006;27:535-543 (zircónia/envelhecimento)</t>
+          <t>Fischer A, Weiß S, Wimmer MA. The tribological difference between biomedical steels and CoCrMo-alloys. J Mech Behav Biomed Mater 2012;9:50-62, Tabela 1</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jmbbm.2012.01.007</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>OBRIGATÓRIO indicar tipo de evidência: in vivo (radiográfico/RSA) vs simulador ISO 14242: não misturar | Iões Co/Cr, ALTR; recolha ASR 2010: candidato a eliminar na triagem</t>
+          <t>varão forjado, não cabeça femoral; HV10 = 340 ± 28 (mín.-máx. = média ± DP); CoCr29Mo6 de baixo carbono, ISO 5832-6 / ASTM F1537, solubilizado | Iões Co/Cr, ALTR; recolha ASR 2010: candidato a eliminar na triagem</t>
         </is>
       </c>
       <c r="N51" t="n">
-        <v>375</v>
+        <v>340</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Monte Carlo com ±10 % nos valores únicos, fontes da fratura cerâmica e do squeaking, Q6 e Q8 do rascunho
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -22471,10 +22471,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
@@ -22511,6 +22511,21 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>incerteza_valor_unico</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Monte Carlo de propriedades: as células quantitativas com mín. = máx. (valor de um único estudo) variam ±10 % à volta do típico; valor de desenho; os ordinais não variam</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Stent, 1.ª ronda: fontes do alongamento, do strut e da reabsorção; métodos passam a usar o valor típico
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:A62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -604,223 +604,230 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.); tipico = ponto médio.</t>
+          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>- Estados da coluna estado:</t>
+          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
+          <t>- Estados da coluna estado:</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
+          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
+          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
-        </is>
-      </c>
+      <c r="A36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
-        </is>
-      </c>
+      <c r="A39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
+          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>- Bioatividade: 5 = liga-se quimicamente ao osso; 4 = osteocondutor; 3 = compósito com fase bioativa; 1 = bioinerte</t>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+          <t>- Bioatividade: 5 = liga-se quimicamente ao osso; 4 = osteocondutor; 3 = compósito com fase bioativa; 1 = bioinerte</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-    </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-    </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Cuidados</t>
-        </is>
-      </c>
+      <c r="A54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade: compara só valores com porosidades semelhantes, ou regista a porosidade.</t>
+          <t>Cuidados</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+          <t>1. Propriedades de scaffolds dependem da porosidade: compara só valores com porosidades semelhantes, ou regista a porosidade.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-    </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Níveis de validação</t>
-        </is>
-      </c>
+      <c r="A60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
+        <is>
+          <t>Níveis de validação</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
         </is>
@@ -6981,22 +6988,32 @@
         </is>
       </c>
       <c r="I94" t="n">
+        <v>40</v>
+      </c>
+      <c r="J94" t="n">
         <v>50</v>
       </c>
-      <c r="J94" t="n">
-        <v>55</v>
-      </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Lamineries Matthey, ficha Alloy L-605 v26E (fita recozida, declara ASTM F90); Fort Wayne Metals, L-605 alloy (fio)</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>https://www.matthey.ch/fileadmin/user_upload/downloads/fichetechnique/EN/Alloy_L-605_v26E.pdf</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>regra da forma: típico = tubo ou fita (forma dos stents, cortados a laser); o fio só alarga o intervalo; típico e mín.: fita recozida A50mm 40 % (Matthey; a ficha não diz se é valor típico ou mínimo de especificação); máx.: fio recozido 50 % (Fort Wayne, valor típico, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); valor anterior: 50-55 % (Hanawa 2009)</t>
         </is>
       </c>
       <c r="N94" t="n">
-        <v>52.5</v>
+        <v>40</v>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -7103,22 +7120,32 @@
         </is>
       </c>
       <c r="I96" t="n">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="J96" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Macaya-Ten F et al. REC Interv Cardiol 2024 (Tabela 3); Brami P et al. J Clin Med 2023</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.24875/RECICE.M24000463</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>XIENCE V / MULTI-LINK VISION: 81 µm; revisões (Brami 2023; Macaya-Ten 2024) que citam o fabricante; espessura de strut = propriedade do dispositivo, não do material; material L-605 confirmado no FDA SSED P070015 (https://www.accessdata.fda.gov/cdrh_docs/pdf7/P070015b.pdf); Brami 2023: https://doi.org/10.3390/jcm12216711; valor anterior: 60-90 µm (Hanawa 2009)</t>
         </is>
       </c>
       <c r="N96" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -7466,22 +7493,32 @@
         </is>
       </c>
       <c r="I102" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J102" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>K-Tube, MP35N Technical Data Sheet (tubo miniatura para stents); Ulbrich, MP35N Wire UNS R30035 (fio, declara ASTM F562)</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>https://www.k-tube.com/wp-content/uploads/2025/12/MP35N-K-Tube-Technical-Data-Sheet.pdf</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>regra da forma: típico = tubo ou fita (forma dos stents, cortados a laser); o fio só alarga o intervalo; típico e mín.: tubo recozido 40 % (K-Tube, tabela "Possible Mechanical Properties": não diz se é típico ou mínimo); máx.: fio recozido 70 % (Ulbrich, valor típico, https://www.ulbrich.com/uploads/data-sheets/MP35N-Wire-UNS-R30035.pdf); valor anterior: 45 % (Hanawa 2009)</t>
         </is>
       </c>
       <c r="N102" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -7588,22 +7625,32 @@
         </is>
       </c>
       <c r="I104" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="J104" t="n">
+        <v>91</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Brami P et al. J Clin Med 2023; Macaya-Ten F et al. REC Interv Cardiol 2024 (Tabela 3)</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/jcm12216711</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>Resolute Integrity 90 µm (Brami 2023); Driver 91 µm (Macaya-Ten 2024); revisões (Brami 2023; Macaya-Ten 2024) que citam o fabricante; espessura de strut = propriedade do dispositivo, não do material; MP35N no Resolute Integrity confirmado no FDA SSED P110013 (https://www.accessdata.fda.gov/cdrh_docs/pdf11/P110013b.pdf); valor anterior: 60-90 µm (Hanawa 2009)</t>
+        </is>
+      </c>
+      <c r="N104" t="n">
         <v>90</v>
       </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
-        </is>
-      </c>
-      <c r="N104" t="n">
-        <v>75</v>
-      </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -8080,15 +8127,25 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Boston Scientific, SYNERGY Product Spec Sheet</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>https://www.bostonscientific.com/content/dam/bostonscientific/Interventional%20Cardiology/portfolio-group/Stents/Synergy/legacy-resource-center/SYNERGY-Product-Spec-Sheet.pdf</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>ficha do fabricante do dispositivo: 74 µm (2,25-2,75 mm), 79 µm (3,00-3,50 mm), 81 µm (4,00 mm); típico = 3,00-3,50 mm; valor anterior: 74-81 µm (Hanawa 2009)</t>
         </is>
       </c>
       <c r="N112" t="n">
-        <v>77.5</v>
+        <v>79</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -9050,7 +9107,17 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Witte F. Acta Biomater 2010;6:1680-1692 (Mg)</t>
+          <t>Rapetto C, Leoncini M. J Thorac Dis 2017 (Tabela 1); Seguchi M et al. EuroIntervention 2023;19:e167</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.21037/jtd.2017.06.34</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>Magmaris: 120 µm (2,5 mm) e 150 µm (3,0-3,5 mm) (Rapetto 2017, revisão); 150 µm no Magmaris de 3,0 mm (Seguchi 2023, estudo pré-clínico, https://doi.org/10.4244/EIJ-D-22-00718); típico = ponto médio; valor anterior: 120-150 µm (Witte 2010)</t>
         </is>
       </c>
       <c r="N128" t="n">
@@ -9058,7 +9125,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -9104,22 +9171,32 @@
         </is>
       </c>
       <c r="I129" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="J129" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Haude M et al. Lancet 2016;387:31-39 (BIOSOLVE-II, Magmaris)</t>
+          <t>Joner M et al. EuroIntervention 2018 (DREAMS 2G/Magmaris, porco); Seguchi M et al. EuroIntervention 2023;19:e167 (pré-clínico, mini-porcos)</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4244/EIJ-D-17-00708</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>modelo animal; todas as fontes são animais; ~1 ano ≈ 95 % reabsorvido (Joner 2018: 94,8 % a 1 ano, só resumo; Seguchi 2023: "approximately 1 year", https://doi.org/10.4244/EIJ-D-22-00718), 2 anos = substituição completa por fosfato de cálcio (Joner 2018); para coerência com o PLLA (reabsorção completa, 36 meses), o típico é o ponto médio; valor anterior: 9-12 meses (Haude 2016, BIOSOLVE-II)</t>
         </is>
       </c>
       <c r="N129" t="n">
-        <v>10.5</v>
+        <v>18</v>
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -9600,7 +9677,17 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Ensaios ABSORB / comunicação FDA 2017 (Absorb BVS)</t>
+          <t>FDA SSED PMA P150023 (Absorb GT1); Gogas BD et al. Int J Cardiovasc Imaging 2012</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>https://www.accessdata.fda.gov/cdrh_docs/pdf15/P150023B.pdf</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>modelo animal (porco): "complete scaffold resorption by approximately 36 months" (SSED, estudos até 42 meses); "At 3 and 4 years ... complete polymer resorption" (Gogas 2012, https://doi.org/10.1007/s10554-011-9860-z); sem fonte humana; valor anterior: 36-48 meses (Ensaios ABSORB / comunicação FDA 2017)</t>
         </is>
       </c>
       <c r="N137" t="n">
@@ -9608,7 +9695,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -21653,7 +21740,7 @@
         <v>0.015</v>
       </c>
       <c r="D6" t="n">
-        <v>0.009833</v>
+        <v>0.008260999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -21669,7 +21756,7 @@
         <v>0.004432</v>
       </c>
       <c r="D7" t="n">
-        <v>0.003883</v>
+        <v>0.003876</v>
       </c>
     </row>
     <row r="8">
@@ -21685,7 +21772,7 @@
         <v>0.022581</v>
       </c>
       <c r="D8" t="n">
-        <v>0.018235</v>
+        <v>0.01791</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Stent, 2.ª ronda: valores de fornecedor do 316L, L605 e MP35N, rubrica e fontes da radiopacidade, densidades; ponto de situação
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A62"/>
+  <dimension ref="A1:A70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -597,222 +597,226 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Legenda</t>
+          <t>Alterações v0.5 (1 out 2026): 2.ª ronda do stent</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.).</t>
+          <t>- Valores de fichas de fornecedor no 316L (alongamento), no L605 (cedência, módulo, tração) e no MP35N (tração), com o valor anterior na nota.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
+          <t>- L605: o típico é o da chapa (Haynes), por não haver ficha de tubo com valores; a fita (Matthey) dá o intervalo.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>- Estados da coluna estado:</t>
+          <t>- Pt-Cr: cedência com fonte primária (O'Brien 2010, só resumo); módulo, tração e alongamento continuam "A verificar", com fontes secundárias na nota.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
+          <t>- Radiopacidade: rubrica escrita (ver "Rubricas ordinais"), fontes nas 7 linhas e estado "Verificado"; as notas não mudam.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
+          <t>- Densidades do 316L, L605, MP35N e Pt-Cr com fonte. A densidade não é critério do stent.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
-        </is>
-      </c>
+      <c r="A32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+          <t>Legenda</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
+          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>- Estados da coluna estado:</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
+          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
+          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
+          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
+          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
-        </is>
-      </c>
+      <c r="A43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>- Bioatividade: 5 = liga-se quimicamente ao osso; 4 = osteocondutor; 3 = compósito com fase bioativa; 1 = bioinerte</t>
+          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
-        </is>
-      </c>
+      <c r="A46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>- Bioatividade: 5 = liga-se quimicamente ao osso; 4 = osteocondutor; 3 = compósito com fase bioativa; 1 = bioinerte</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cuidados</t>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade: compara só valores com porosidades semelhantes, ou regista a porosidade.</t>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
         </is>
       </c>
     </row>
@@ -822,12 +826,60 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Cuidados</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1. Propriedades de scaffolds dependem da porosidade: compara só valores com porosidades semelhantes, ou regista a porosidade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>Níveis de validação</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
+    <row r="70">
+      <c r="A70" t="inlineStr">
         <is>
           <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
         </is>
@@ -6506,19 +6558,29 @@
         <v>40</v>
       </c>
       <c r="J86" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Alleima, ficha 316LVM (tubo de parede fina recozido); patente US 6780261 B2 (Scimed), tubo de stent totalmente recozido</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>https://patents.google.com/patent/US6780261B2/en</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>típico e mín.: tubo de parede fina recozido 40 % (Alleima 316LVM, coluna "typical", não é mínimo de especificação); máx.: tubo de stent totalmente recozido ~50 % (patente US 6780261 B2, Scimed); valor anterior: 40-60 % (Hanawa T. J Artif Organs 2009;12:73-79); o doi_url é o da patente (fonte do máx.); ficha da Alleima sem URL registado</t>
         </is>
       </c>
       <c r="N86" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -6571,7 +6633,12 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Alleima, ficha 316LVM</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>valor anterior: 8 g/cm³ (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N87" t="n">
@@ -6579,7 +6646,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -6800,27 +6867,32 @@
         </is>
       </c>
       <c r="I91" t="n">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="J91" t="n">
         <v>243</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Lamineries Matthey, ficha Alloy L-605 v26E (fita recozida, declara ASTM F90); Haynes International, HAYNES 25 (chapa solubilizada); Fort Wayne Metals, L-605 alloy (barra e fio)</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>https://www.matthey.ch/fileadmin/user_upload/downloads/fichetechnique/EN/Alloy_L-605_v26E.pdf</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>Slides: F90 (Co-Cr-W-Ni)</t>
+          <t>Slides: F90 (Co-Cr-W-Ni); Matthey e Haynes 225 GPa; Fort Wayne 243 GPa (https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); típico da chapa (Haynes) por não haver ficha de tubo com valores; a fita (Matthey) dá o intervalo; valor anterior: 243 GPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N91" t="n">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -6866,22 +6938,32 @@
         </is>
       </c>
       <c r="I92" t="n">
-        <v>460</v>
+        <v>380</v>
       </c>
       <c r="J92" t="n">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Lamineries Matthey, ficha Alloy L-605 v26E (fita recozida, declara ASTM F90); Haynes International, HAYNES 25 (chapa solubilizada); Fort Wayne Metals, L-605 alloy (barra e fio)</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>https://www.matthey.ch/fileadmin/user_upload/downloads/fichetechnique/EN/Alloy_L-605_v26E.pdf</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>intervalo: fita recozida 380-700 MPa (Matthey); típico: chapa solubilizada 476 MPa (Haynes); barra 517 MPa e fio 621 MPa (Fort Wayne, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy) dentro do intervalo; típico da chapa (Haynes) por não haver ficha de tubo com valores; a fita (Matthey) dá o intervalo; valor anterior: 460-500 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N92" t="n">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -6927,22 +7009,32 @@
         </is>
       </c>
       <c r="I93" t="n">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="J93" t="n">
-        <v>1050</v>
+        <v>1138</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Lamineries Matthey, ficha Alloy L-605 v26E (fita recozida, declara ASTM F90); Haynes International, HAYNES 25 (chapa solubilizada); Fort Wayne Metals, L-605 alloy (barra e fio)</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>https://www.matthey.ch/fileadmin/user_upload/downloads/fichetechnique/EN/Alloy_L-605_v26E.pdf</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>fita recozida 900-1000 MPa (Matthey); chapa 996 MPa (Haynes); fio 1138 MPa (Fort Wayne, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); típico da chapa (Haynes) por não haver ficha de tubo com valores; a fita (Matthey) dá o intervalo; valor anterior: 1000-1050 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N93" t="n">
-        <v>1025</v>
+        <v>996</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -7059,22 +7151,32 @@
         </is>
       </c>
       <c r="I95" t="n">
-        <v>9.1</v>
+        <v>9.07</v>
       </c>
       <c r="J95" t="n">
-        <v>9.1</v>
+        <v>9.27</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Lamineries Matthey, ficha Alloy L-605 v26E (fita); Haynes International, HAYNES 25</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>https://www.matthey.ch/fileadmin/user_upload/downloads/fichetechnique/EN/Alloy_L-605_v26E.pdf</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>mín.: 9,07 g/cm³ (Haynes, HAYNES 25, https://haynesintl.com/en/alloys/alloy-portfolio/high-temperature-alloys/haynes-25/); típico e máx.: 9,27 g/cm³ (Matthey, fita); valor anterior: 9,1 g/cm³ (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N95" t="n">
-        <v>9.1</v>
+        <v>9.27</v>
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -7432,22 +7534,32 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="J101" t="n">
-        <v>960</v>
+        <v>965</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>K-Tube, MP35N Technical Data Sheet (tubo miniatura para stents); Ulbrich, MP35N Wire UNS R30035 (fio, declara ASTM F562)</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>https://www.k-tube.com/wp-content/uploads/2025/12/MP35N-K-Tube-Technical-Data-Sheet.pdf</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>típico e máx.: tubo recozido 140 ksi = 965 MPa (K-Tube; conversão 1 ksi = 6,895 MPa); mín.: fio 931 MPa (Ulbrich, https://www.ulbrich.com/uploads/data-sheets/MP35N-Wire-UNS-R30035.pdf); valor anterior: 930-960 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N101" t="n">
-        <v>945</v>
+        <v>965</v>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -7564,22 +7676,32 @@
         </is>
       </c>
       <c r="I103" t="n">
-        <v>8.4</v>
+        <v>8.43</v>
       </c>
       <c r="J103" t="n">
-        <v>8.4</v>
+        <v>8.43</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Ulbrich, MP35N Wire UNS R30035 (declara ASTM F562)</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>https://www.ulbrich.com/uploads/data-sheets/MP35N-Wire-UNS-R30035.pdf</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>valor anterior: 8,4 g/cm³ (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N103" t="n">
-        <v>8.4</v>
+        <v>8.43</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7944,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>Alta radiopacidade</t>
+          <t>Alta radiopacidade; fontes secundárias, valor ainda não confirmado na fonte original: Huibregtse &amp; Granada 2011 (Cardiac Interventions Today); Samant 2021 (Sci Rep, suplemento)</t>
         </is>
       </c>
       <c r="N107" t="n">
@@ -7883,7 +8005,17 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>O'Brien BJ, Stinson JS, Larsen SR, Eppihimer MJ, Carroll WM. A platinum-chromium steel for cardiovascular stents. Biomaterials 2010;31:3755-3761</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.biomaterials.2010.01.146</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>só resumo; valor anterior: 480 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N108" t="n">
@@ -7891,7 +8023,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -7947,6 +8079,11 @@
           <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
         </is>
       </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>fontes secundárias, valor ainda não confirmado na fonte original: Huibregtse &amp; Granada 2011 (Cardiac Interventions Today); Samant 2021 (Sci Rep, suplemento)</t>
+        </is>
+      </c>
       <c r="N109" t="n">
         <v>834</v>
       </c>
@@ -8008,6 +8145,11 @@
           <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
         </is>
       </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>fontes secundárias, valor ainda não confirmado na fonte original: Huibregtse &amp; Granada 2011 (Cardiac Interventions Today); Samant 2021 (Sci Rep, suplemento)</t>
+        </is>
+      </c>
       <c r="N110" t="n">
         <v>45</v>
       </c>
@@ -8066,7 +8208,17 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324)</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>valor anterior: 9,9 g/cm³ (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N111" t="n">
@@ -8074,7 +8226,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -16828,12 +16980,17 @@
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>Radiopacidade depende sobretudo do número atómico efetivo e da espessura: confirmar com literatura de stents</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>Visibilidade reduzida com struts finos</t>
+          <t>Visibilidade reduzida com struts finos; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N247" t="n">
@@ -16841,7 +16998,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -16894,12 +17051,17 @@
       </c>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Radiopacidade depende sobretudo do número atómico efetivo e da espessura: confirmar com literatura de stents</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>W na liga aumenta a radiopacidade</t>
+          <t>W na liga aumenta a radiopacidade; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N248" t="n">
@@ -16907,7 +17069,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -16960,7 +17122,17 @@
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>Radiopacidade depende sobretudo do número atómico efetivo e da espessura: confirmar com literatura de stents</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N249" t="n">
@@ -16968,7 +17140,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -17021,12 +17193,17 @@
       </c>
       <c r="K250" t="inlineStr">
         <is>
-          <t>Radiopacidade depende sobretudo do número atómico efetivo e da espessura: confirmar com literatura de stents</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>Pt: número atómico elevado</t>
+          <t>Pt: número atómico elevado; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N250" t="n">
@@ -17034,7 +17211,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -17087,12 +17264,17 @@
       </c>
       <c r="K251" t="inlineStr">
         <is>
-          <t>Radiopacidade depende sobretudo do número atómico efetivo e da espessura: confirmar com literatura de stents</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>Precisa de marcadores</t>
+          <t>Precisa de marcadores; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N251" t="n">
@@ -17100,7 +17282,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -17153,12 +17335,17 @@
       </c>
       <c r="K252" t="inlineStr">
         <is>
-          <t>Radiopacidade depende sobretudo do número atómico efetivo e da espessura: confirmar com literatura de stents</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>Precisa de marcadores radiopacos</t>
+          <t>Precisa de marcadores radiopacos; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N252" t="n">
@@ -17166,7 +17353,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -17219,12 +17406,17 @@
       </c>
       <c r="K253" t="inlineStr">
         <is>
-          <t>Radiopacidade depende sobretudo do número atómico efetivo e da espessura: confirmar com literatura de stents</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>Marcadores de Pt nas extremidades</t>
+          <t>Marcadores de Pt nas extremidades; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N253" t="n">
@@ -17232,7 +17424,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -21686,13 +21878,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.001893</v>
+        <v>0.001564</v>
       </c>
       <c r="C3" t="n">
-        <v>0.002058</v>
+        <v>0.003111</v>
       </c>
       <c r="D3" t="n">
-        <v>0.001975</v>
+        <v>0.002116</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Scaffold, 1.ª ronda: fontes primárias em 12 linhas, rubrica da bioatividade segundo Hench e regra da porosidade
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A70"/>
+  <dimension ref="A1:A76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -642,229 +642,229 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Legenda</t>
+          <t>Alterações v0.6 (1 out 2026): 1.ª ronda do scaffold</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.).</t>
+          <t>- Rubrica da bioatividade reescrita segundo a classificação de Hench (classes A e B); as notas dos materiais não mudam.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
+          <t>- Regra da porosidade para as propriedades mecânicas dos scaffolds (ver "Cuidados").</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>- Estados da coluna estado:</t>
+          <t>- 11 linhas do scaffold com fonte primária: porosidade do quitosano/HA, do PLLA e do β-TCP; resistência à compressão da HA; e sete notas ordinais (imprimibilidade, esterilização e bioatividade).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
+          <t>- A esterilização da HA continua "A verificar".</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
-        </is>
-      </c>
+      <c r="A38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
+          <t>Legenda</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
+          <t>- Estados da coluna estado:</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
+          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
+          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
+          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
-        </is>
-      </c>
+      <c r="A49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
+          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>- Bioatividade: 5 = liga-se quimicamente ao osso; 4 = osteocondutor; 3 = compósito com fase bioativa; 1 = bioinerte</t>
-        </is>
-      </c>
+      <c r="A52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
+          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr"/>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Cuidados</t>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade: compara só valores com porosidades semelhantes, ou regista a porosidade.</t>
+          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
-        </is>
-      </c>
+      <c r="A66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
         </is>
       </c>
     </row>
@@ -874,12 +874,50 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Níveis de validação</t>
+          <t>Cuidados</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
+        <is>
+          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Regista sempre a porosidade e o método de fabrico do estudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Níveis de validação</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
         <is>
           <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
         </is>
@@ -10485,12 +10523,17 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
+          <t>Lu L et al. Biomaterials 2000;21:1595-1605; Budyanto L, Goh YQ, Ooi CP. J Mater Sci Mater Med 2009;20:105-111; Ghosh S et al. J Mater Sci Mater Med 2007;18:185-193</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/S0142-9612(00)00048-X</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+          <t>só resumo (as três fontes): 67-91 % por lixiviação de sal (Lu 2000); 80-90 % por separação de fases (Budyanto 2009, https://doi.org/10.1007/s10856-008-3545-8); 76-86 % por moldação com dois porogénios (Ghosh 2007, https://doi.org/10.1007/s10856-006-0680-y); o mínimo de 60 % não tem fonte; fonte anterior: Karageorgiou &amp; Kaplan 2005; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N147" t="n">
@@ -10498,7 +10541,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -11138,27 +11181,32 @@
         </is>
       </c>
       <c r="I157" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="J157" t="n">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Liang H et al. Int J Bioprint 2022;8(1):502; Zhang P, Zhou Q, He R. Materials 2024;17:6092 (Tabela 1)</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.18063/ijb.v8i1.502</t>
         </is>
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>regra da porosidade (típico da HA: 65 %, janela 55-75 %): a ~70 % de porosidade, 3,4 MPa (BCC), 5,9 MPa (TPMS-P) e 22,5 MPa (poros cúbicos), DLP e sinterização a 1250 °C (Liang 2022, texto completo); a 60 %, 1,59-3,32 MPa (Zhang 2024, Tabela 1, texto completo, https://doi.org/10.3390/ma17246092); típico = estrutura BCC a ~70 %; de fora: 0,09-0,50 MPa a 80 % e 12,1-19,2 MPa a 40 % (Zhang 2024); são redes impressas, não espumas; valor anterior: 2-20 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N157" t="n">
-        <v>11</v>
+        <v>3.4</v>
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -11409,12 +11457,17 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
+          <t>Grandfield K et al. J R Soc Interface 2010;7:1497-1501; rubrica segundo a classificação de Hench (LEIA-ME)</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1098/rsif.2010.0213</t>
         </is>
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>nota 4 pela rubrica (classe B de Hench, osteocondutor com ligação ao osso): scaffold de HA porosa em mandíbula humana, apatite precipitada na interface (Grandfield 2010; página de texto completo lida por extração automática, confirmar no PDF); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N161" t="n">
@@ -11422,7 +11475,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -11666,19 +11719,24 @@
         </is>
       </c>
       <c r="I165" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="J165" t="n">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
+          <t>FDA 510(k) K120152 (Cerasorb Plus); FDA 510(k) K032409 (Vitoss); Furusawa T et al. Int J Implant Dent 2016;2:4</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>https://fda.innolitics.com/device/K120152</t>
         </is>
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>típico e mín.: Cerasorb Plus em bloco, 65 %; Vitoss cerca de 90 % (https://fda.innolitics.com/device/K032409); máx.: 92 % por espumação e liofilização (Furusawa 2016, Tabela 1, https://doi.org/10.1186/s40729-016-0037-3); o Cerasorb Plus de 35 % fica de fora: outra forma de produto; 510(k) lidos numa cópia de terceiros; valor anterior: 50-80 % (Karageorgiou V, Kaplan D. Biomaterials 2005;26); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N165" t="n">
@@ -11686,7 +11744,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -11805,12 +11863,17 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
+          <t>Kotani S et al. J Biomed Mater Res 1991;25:1303-1315; rubrica segundo a classificação de Hench (LEIA-ME)</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jbm.820251010</t>
         </is>
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>só resumo: β-TCP denso em tíbia de coelho liga-se ao osso sem camada de apatite (Kotani 1991); nota 4 pela rubrica (classe B, osteocondutor); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N167" t="n">
@@ -11818,7 +11881,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -12597,12 +12660,17 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
+          <t>Bruyas A et al. J Mater Res 2018;33:1948-1959; rubrica segundo a classificação de Hench (LEIA-ME)</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1557/jmr.2018.112</t>
         </is>
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>nota 3 pela rubrica (compósito com fase bioativa): mais células e mais atividade de ALP com β-TCP, in vitro (Bruyas 2018, FDM com 0-60 % de β-TCP; página de texto completo lida por extração automática); Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N179" t="n">
@@ -12610,7 +12678,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -12854,19 +12922,24 @@
         </is>
       </c>
       <c r="I183" t="n">
-        <v>80</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="J183" t="n">
-        <v>95</v>
+        <v>91.3</v>
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
+          <t>Gaihre B, Jayasuriya AC. Mater Sci Eng C 2018;91:330-339; Wang H et al. Heliyon 2024;10:e25832</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.msec.2018.05.060</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: fonte a indicar</t>
+          <t>típico: 87,5 ± 11,2 % (Gaihre 2018, quitosano com 40 % de nHA, liofilizado, deslocamento de etanol; texto completo); intervalo: 86,9-91,3 % com 1-4 % de HAp, liofilizado (Wang 2024, Fig. 3a, https://doi.org/10.1016/j.heliyon.2024.e25832); valor anterior: 80-95 % (Karageorgiou V, Kaplan D. Biomaterials 2005;26); Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N183" t="n">
@@ -12874,7 +12947,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -13059,12 +13132,17 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
+          <t>Bergonzi C et al. Sci Rep 2019;9:362</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41598-018-36613-8</t>
         </is>
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: fonte a indicar</t>
+          <t>nota 2 pela rubrica: o material é liofilizado; a impressão de quitosano exige técnica especial (deposição sobre superfície arrefecida e gelificação em banho; Bergonzi 2019, quitosano sem HA, texto completo); Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N186" t="n">
@@ -13072,7 +13150,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -19381,12 +19459,17 @@
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Holy CE, Cheng C, Davies JE, Shoichet MS. Biomaterials 2001;22:25-31 (Tabela 2)</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/S0142-9612(00)00136-8</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>Muito sensível: altera a degradação; Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+          <t>nota 2 pela rubrica (degradação documentada): gama 2,5 Mrad, Mw -54 %; EtO, Mw -12 % e volume -50 % (Holy 2001, texto completo); a fonte usa scaffolds de PLGA 75/25, não 50:50, e não indica a porosidade; Muito sensível: altera a degradação; Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
         </is>
       </c>
       <c r="N283" t="n">
@@ -19394,7 +19477,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -19452,7 +19535,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>Autoclave/calor seco; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>a confirmar: o autoclave (121 °C, 40 min) altera a dissolubilidade, a resistência e a morfologia da HA porosa (Li X et al. J Mater Sci Mater Med 2016;27:5, https://doi.org/10.1007/s10856-015-5617-x, só resumo); falta fonte para radiação gama em HA; Autoclave/calor seco; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N284" t="n">
@@ -19513,12 +19596,17 @@
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>FDA 510(k) K032409 (Vitoss, Orthovita, 2003); FDA 510(k) K120152 (Cerasorb Plus, Riemser, 2012)</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>https://fda.innolitics.com/device/K032409</t>
         </is>
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>nota 5 pela rubrica: os dois produtos são esterilizados por radiação gama (resumos dos 510(k), lidos numa cópia de terceiros, https://fda.innolitics.com/device/K120152); ressalva: o autoclave altera a morfologia e a resistência do β-TCP poroso (Li X et al. J Mater Sci Mater Med 2016;27:5, https://doi.org/10.1007/s10856-015-5617-x, só resumo); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N285" t="n">
@@ -19526,7 +19614,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -19645,12 +19733,17 @@
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Bruyas A et al. Tissue Eng Part A 2019;25:248-256</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1089/ten.tea.2018.0130</t>
         </is>
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>Limitado pela fase PCL; Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>nota 3 pela rubrica (método restrito com risco de degradação): scaffolds PCL/β-TCP por FDM, feixe de eletrões: +14 % de rigidez e resistência iniciais e degradação 25 % mais rápida (Bruyas 2019, só resumo); o calor está excluído pela fusão do PCL; Limitado pela fase PCL; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N287" t="n">
@@ -19658,7 +19751,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stent: fontes das frases por confirmar, espessura de strut do 316L e normas com edição
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -6730,22 +6730,32 @@
         </is>
       </c>
       <c r="I88" t="n">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="J88" t="n">
         <v>140</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
+          <t>Nikam N, Steinberg TB, Steinberg DH. Med Devices (Auckl) 2014;7:165-178 (Tabela 1)</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2147/MDER.S31869</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>revisão, texto completo: plataformas de 316L de primeira geração, Express 132 µm e Bx Velocity (Cypher) 140 µm; Multi-Link Duet 140 µm no ISAR-STEREO (Kastrati 2001, https://doi.org/10.1161/01.CIR.103.23.2816); típico = ponto médio; espessura de strut = propriedade do dispositivo, não do material; o 316L também existiu com struts finos (Multi-Link 50 µm, Liberté 81 µm); valor anterior: 100-140 µm (Hanawa T. J Artif Organs 2009;12)</t>
         </is>
       </c>
       <c r="N88" t="n">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scaffold, 2.ª ronda: valores mecânicos, degradação e porosidades com fonte; regra da mediana na janela de porosidade
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A76"/>
+  <dimension ref="A1:A85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -680,244 +680,303 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Legenda</t>
+          <t>Alterações v0.7 (1 out 2026): 2.ª ronda do scaffold</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.).</t>
+          <t>- Regra do típico: típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
+          <t>- β-TCP: resistência 0,35-7,72 MPa, típico 2. PCL/β-TCP: porosidade típica 70 % (especificação dos scaffolds por FDM).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>- Estados da coluna estado:</t>
+          <t>- HA: tempo de degradação tratado como não reabsorvível (mínimo 42 meses; máximo e típico = pior valor observado nos outros materiais, como a opção O2 do stent).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
+          <t>- PLLA definido como scaffold impresso; degradação 24-60 meses, com dados de PLLA maciço.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
+          <t>- Vidro 45S5: resistência 0,2-1,1 MPa e degradação 6-24 meses (dados de partículas). O módulo fica sem fonte primária.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
+          <t>- Quitosano/HA: módulo e resistência cerca de dez vezes abaixo dos valores anteriores.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+          <t>- Porosidades do PCL, do PLGA e da HA com fonte.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
-        </is>
-      </c>
+      <c r="A47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
+          <t>Legenda</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.).</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
+          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
+          <t>- Estados da coluna estado:</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
+          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
+          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
+          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
+          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
-        </is>
-      </c>
+      <c r="A58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
-        </is>
-      </c>
+      <c r="A61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
+          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr"/>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Cuidados</t>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Regista sempre a porosidade e o método de fabrico do estudo.</t>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Níveis de validação</t>
-        </is>
-      </c>
+      <c r="A75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
+        <is>
+          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Cuidados</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Dentro da janela, típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes. Regista sempre a porosidade e o método de fabrico do estudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Níveis de validação</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
         <is>
           <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
         </is>
@@ -10130,27 +10189,32 @@
         </is>
       </c>
       <c r="I141" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J141" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
+          <t>Zein I et al. Biomaterials 2002;23:1169-1185; Hutmacher DW et al. J Biomed Mater Res 2001;55:203-216</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/s0142-9612(01)00232-0</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+          <t>FDM de PCL: 48-77 % (Zein 2002); 61 ± 1 % (Hutmacher 2001); só resumo nos dois; valor anterior: 50-80 % (Karageorgiou V, Kaplan D. Biomaterials 2005;26); Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
         </is>
       </c>
       <c r="N141" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -10401,20 +10465,25 @@
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Karanth D et al. Clin Exp Dent Res 2023;9:398-408</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/cre2.712</t>
         </is>
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+          <t>definido como scaffold impresso ou extrudido (filamentos densos), não espuma: 5,06 ± 1,48 MPa a 73 % de porosidade (Karanth 2023, FDM, texto completo); uma só fonte; o intervalo 1-10 MPa vem do valor anterior; valor anterior: 1-10 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N145" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -10467,12 +10536,17 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Karanth D et al. Clin Exp Dent Res 2023;9:398-408; Yin HM et al. Polymers 2016;8:213</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/cre2.712</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+          <t>definido como scaffold impresso ou extrudido (filamentos densos), não espuma: 244 MPa a 73 % de porosidade (Karanth 2023, FDM); 86-207 MPa a 66-81 % (Yin 2016, extrusão e lixiviação, https://doi.org/10.3390/polym8060213; o artigo diz PLA sem indicar o grau); texto completo nos dois; espumas por separação de fases ou lixiviação de sal têm 3-35 MPa e ficam de fora; fonte anterior: Rezwan 2006; Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N146" t="n">
@@ -10480,7 +10554,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -10597,27 +10671,32 @@
         </is>
       </c>
       <c r="I148" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="J148" t="n">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Bos RRM et al. Biomaterials 1991;12:32-36; Bergsma JE et al. Biomaterials 1995;16:25-31</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/0142-9612(91)90128-w</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+          <t>dados de PLLA maciço (Bos 1991, rato, reabsorção não completa aos 3 anos; Bergsma 1995, humanos, partículas ainda presentes aos 5,7 anos, https://doi.org/10.1016/0142-9612(95)91092-d; só resumo nos dois); o scaffold poroso pode degradar-se mais depressa; típico = ponto médio; valor anterior: 18-36 meses (Rezwan K et al. Biomaterials 2006;27); Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N148" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -10927,19 +11006,24 @@
         </is>
       </c>
       <c r="I153" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="J153" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
+          <t>Lu L et al. Biomaterials 2000;21:1837-1845</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/s0142-9612(00)00047-8</t>
         </is>
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+          <t>espumas por lixiviação de sal: 73, 84 e 87 % (Lu 2000, só resumo); típico = ponto médio; valor anterior: 70-90 % (Karageorgiou V, Kaplan D. Biomaterials 2005;26); Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
         </is>
       </c>
       <c r="N153" t="n">
@@ -10947,7 +11031,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -11328,19 +11412,24 @@
         </is>
       </c>
       <c r="I159" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="J159" t="n">
         <v>80</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
+          <t>FDA 510(k) K023998 (Tabela 1: Pro Osteon 200); Hoogendoorn HA et al. Clin Orthop Relat Res 1984;187:281-288</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>https://www.accessdata.fda.gov/cdrh_docs/pdf2/K023998.pdf</t>
         </is>
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>Pro Osteon 200 (HA coralina): porosidade 57 %, resistência à compressão 5,8 MPa (4-10 MPa), conferido no PDF do 510(k); blocos sinterizados com 56 % de macroporosidade (Hoogendoorn 1984, só resumo); o típico de 65 % e o máximo de 80 % não têm fonte própria; valor anterior: 50-80 % (Karageorgiou V, Kaplan D. Biomaterials 2005;26); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N159" t="n">
@@ -11348,7 +11437,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -11394,27 +11483,32 @@
         </is>
       </c>
       <c r="I160" t="n">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="J160" t="n">
         <v>60</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Hoogendoorn HA et al. Clin Orthop Relat Res 1984;187:281-288; Oonishi H et al. J Biomed Mater Res 2000;51:37-46</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1097/00003086-198407000-00043</t>
         </is>
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>não reabsorvível; valor de modelação, como a opção O2 do stent: mínimo 42 meses (sem reabsorção mensurável em 3,5 anos, cão, blocos com 56 % de macroporosidade, Hoogendoorn 1984; "not resorbed at all", coelho, Oonishi 2000; só resumo nos dois); máximo e típico = pior valor observado nos outros materiais do scaffold (60 meses, PLLA); valor anterior: 24-60 meses (Rezwan K et al. Biomaterials 2006;27); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N160" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -11597,27 +11691,32 @@
         </is>
       </c>
       <c r="I163" t="n">
-        <v>1</v>
+        <v>0.35</v>
       </c>
       <c r="J163" t="n">
-        <v>15</v>
+        <v>7.72</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Montelongo SA et al. J Mater Sci Mater Med 2021;32:94; Xulin H et al. Int J Bioprint 2023;9(2):673; Hashimoto K, Oikawa H, Shibata H. Int J Mol Sci 2024;25:5363</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10856-021-06569-9</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>regra da porosidade (típico do β-TCP: 65 %, janela 55-75 %), típico = mediana das três fontes: 7,72 MPa a 59,6 % (Montelongo 2021, impressão 3D e sinterização); 0,35 MPa a 66 % (Xulin 2023, impressão por gel, https://doi.org/10.18063/ijb.v9i2.673); cerca de 2 MPa a ~70 % (Hashimoto 2024, espumação e liofilização, valor aproximado do texto, exato só em figura, https://doi.org/10.3390/ijms25105363); texto completo nas três; de fora: 0,45 MPa a 92 % (Furusawa 2016) e 72 MPa a 35 % (Esslinger 2021); valor anterior: 1-15 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N163" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -11675,7 +11774,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>uma só fonte na janela de porosidade: 546 MPa a 59,6 % (Montelongo 2021, texto completo, https://doi.org/10.1007/s10856-021-06569-9); o intervalo 100-1000 MPa continua a vir da revisão; Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N164" t="n">
@@ -12003,27 +12102,32 @@
         </is>
       </c>
       <c r="I169" t="n">
-        <v>0.3</v>
+        <v>0.58</v>
       </c>
       <c r="J169" t="n">
-        <v>2</v>
+        <v>1.1</v>
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>Hench LL. J Am Ceram Soc 1991;74:1487-1510 (vidros bioativos)</t>
+          <t>Baino F, Fiume E. Materials 2019;12:3244 (Tabela 1)</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma12193244</t>
         </is>
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+          <t>regra da porosidade (típico do 45S5: 80 %, janela 70-90 %), típico = mediana dos seis valores da Tabela 1 na janela: 0,58 MPa a 86 %, 0,78 a 82 %, 0,88 a 80 %, 0,95 a 75 %, 0,96 a 71 % e 1,1 a 70 % (Baino e Fiume 2019, espumas por réplica de esponja, texto completo); valor anterior: 0,3-2 MPa (Hench LL. J Am Ceram Soc 1991;74); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
         </is>
       </c>
       <c r="N169" t="n">
-        <v>1.15</v>
+        <v>0.915</v>
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -12081,7 +12185,7 @@
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+          <t>sem fonte primária: Baino e Fiume 2019 dão 1,2-8 GPa, mas é módulo elástico dinâmico (excitação por impulso), não o módulo do ensaio de compressão, por isso não se aplica; Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
         </is>
       </c>
       <c r="N170" t="n">
@@ -12204,24 +12308,29 @@
         <v>6</v>
       </c>
       <c r="J172" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>Hench LL. J Am Ceram Soc 1991;74:1487-1510 (vidros bioativos)</t>
+          <t>Tadjoedin ES et al. Clin Oral Implants Res 2002;13:428-436; Tadjoedin ES et al. Clin Oral Implants Res 2000;11:334-344</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1034/j.1600-0501.2002.130412.x</t>
         </is>
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+          <t>partículas, não scaffold (Tadjoedin 2000, 2002): em seio maxilar humano, 8 % do volume de vidro aos 15 meses e desaparecimento aos 16 meses; só resumo; o resumo não diz que o BioGran é 45S5 (a confirmar); valor anterior: 6-12 meses (Hench LL. J Am Ceram Soc 1991;74); Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
         </is>
       </c>
       <c r="N172" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -12399,23 +12508,28 @@
         </is>
       </c>
       <c r="I175" t="n">
-        <v>3</v>
+        <v>2.2</v>
       </c>
       <c r="J175" t="n">
-        <v>12</v>
+        <v>6.38</v>
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Kawai T et al. J Orthop Res 2018;36:1002-1011; Wong WS et al. Cureus 2025;17:e86272</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jor.23673</t>
         </is>
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>regra da porosidade (típico do PCL/β-TCP: 70 %, janela 60-80 %), PCL/TCP 80:20 por FDM ou extrusão: a verificar, duas fontes fracas: 2,2 MPa a 59,5 %, no limite inferior da janela (Kawai 2018, texto completo); 6,38 MPa a 70 % (Wong 2025, fonte secundária, https://doi.org/10.7759/cureus.86272); típico = ponto médio; de fora: 27,9 MPa em Wang 2024, que não é tensão de cedência; valor anterior: 3-12 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N175" t="n">
-        <v>7.5</v>
+        <v>4.3</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
@@ -12465,27 +12579,32 @@
         </is>
       </c>
       <c r="I176" t="n">
-        <v>30</v>
+        <v>22.2</v>
       </c>
       <c r="J176" t="n">
-        <v>150</v>
+        <v>51.5</v>
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Reichert JC et al. Int Orthop 2011;35:1229-1236; Wang Y et al. Heliyon 2024;10:e26071 (Tabela 3); Kawai T et al. J Orthop Res 2018;36:1002-1011</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s00264-010-1146-x</t>
         </is>
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>regra da porosidade (típico do PCL/β-TCP: 70 %, janela 60-80 %), PCL/TCP 80:20 por FDM ou extrusão, típico = mediana de quatro valores: 22,2 MPa a 70,6 % em PBS (Reichert 2011, mPCL-TCP); 48,2 MPa a 65,1 % (Wang 2024, https://doi.org/10.1016/j.heliyon.2024.e26071); 51,5 MPa a 59,5 % (Kawai 2018, https://doi.org/10.1002/jor.23673); 23,1 MPa a 70 % (Wong 2025, fonte secundária, https://doi.org/10.7759/cureus.86272); texto completo em todas; valor anterior: 30-150 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N176" t="n">
-        <v>90</v>
+        <v>35.7</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -12531,27 +12650,32 @@
         </is>
       </c>
       <c r="I177" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="J177" t="n">
         <v>70</v>
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>Karageorgiou V, Kaplan D. Biomaterials 2005;26:5474-5491 (porosidade)</t>
+          <t>Sparks DS et al. Sci Adv 2023;9:eadd6071; Nam JH et al. J Periodontal Implant Sci 2023;53:218-232</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1126/sciadv.add6071</t>
         </is>
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>regra da forma: especificação dos scaffolds mPCL-TCP (80:20) por FDM, 70 % de porosidade (Sparks 2023; Nam 2023, micro-CT, https://doi.org/10.5051/jpis.2300660033; texto completo nos dois); é valor de especificação repetido em vários artigos, não uma tabela de medições; o mínimo de 60 % vem do valor anterior; valor anterior: 50-70 % (Karageorgiou V, Kaplan D. Biomaterials 2005;26); Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N177" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -12609,7 +12733,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>a verificar: as fontes divergem e nenhuma mede a reabsorção completa (Yeo 2008, rato, 24 semanas, Mw -89 %; Lam 2009, coelho, 6 meses, perda de massa de cerca de 7 %; só resumo nos dois); Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N178" t="n">
@@ -12800,27 +12924,32 @@
         </is>
       </c>
       <c r="I181" t="n">
-        <v>0.1</v>
+        <v>0.03</v>
       </c>
       <c r="J181" t="n">
-        <v>1</v>
+        <v>0.06</v>
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Gaihre B, Jayasuriya AC. Mater Sci Eng C 2018;91:330-339</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.msec.2018.05.060</t>
         </is>
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte a indicar</t>
+          <t>uma só fonte: 0,050-0,055 MPa seco a 87,5 % nos compósitos e 0,028 MPa no quitosano puro (Gaihre 2018, texto completo; o valor exato do compósito com nHA está só em figura); valor anterior: 0,1-1 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N181" t="n">
-        <v>0.55</v>
+        <v>0.05</v>
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -12866,27 +12995,32 @@
         </is>
       </c>
       <c r="I182" t="n">
-        <v>1</v>
+        <v>0.08</v>
       </c>
       <c r="J182" t="n">
-        <v>10</v>
+        <v>0.8</v>
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Gaihre B, Jayasuriya AC. Mater Sci Eng C 2018;91:330-339; Wang H et al. Heliyon 2024;10:e25832</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.msec.2018.05.060</t>
         </is>
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t>Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte a indicar</t>
+          <t>regra da porosidade (janela 77,5-97,5 %): 0,76 MPa seco a 87,5 % (Gaihre 2018, texto completo); 0,076 MPa hidratado a 89,8 % (Wang 2024, texto completo, https://doi.org/10.1016/j.heliyon.2024.e25832); típico = valor seco; valor anterior: 1-10 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N182" t="n">
-        <v>5.5</v>
+        <v>0.76</v>
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -13015,7 +13149,7 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: fonte a indicar</t>
+          <t>a verificar: só há dados in vitro (perda de massa de 1-4 % num mês com lisozima, Reves 2012, texto completo, https://doi.org/10.3390/jfb3010114); sem tempo de reabsorção in vivo; Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N184" t="n">
@@ -19682,7 +19816,7 @@
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+          <t>calor seco; a radiação gama aumenta a dissolução (Farag 2017, só resumo, https://doi.org/10.1002/jbm.a.36035); Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
         </is>
       </c>
       <c r="N286" t="n">

</xml_diff>

<commit_message>
Stent: regra da forma revista (intervalo só com a forma do dispositivo)
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A85"/>
+  <dimension ref="A1:A90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -739,244 +739,275 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Legenda</t>
+          <t>Alterações v0.8 (2 out 2026): regra da forma revista (stent)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.).</t>
+          <t>- Regra da forma: nas propriedades dependentes da forma do produto, min, max e tipico cobrem só a forma usada no dispositivo (no stent: tubo ou fita); os valores de outras formas (fio, barra, chapa) ficam só na coluna notas. Se a forma do dispositivo tiver um único valor, min = max e o Monte Carlo aplica ±10 % (incerteza_valor_unico em parametros.csv).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
+          <t>- Linhas revistas: L605 módulo 225 (antes 225-243), tração 900-1000 (antes 900-1138), alongamento 40 (antes 40-50); MP35N tração 965 (antes 931-965), alongamento 40 (antes 40-70). Sem alteração: 316L alongamento 40-50 e L605 cedência 380-700. Os típicos não mudaram.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>- Estados da coluna estado:</t>
+          <t>- Exceção mantida no L605: o típico da cedência e da tração é o da chapa (Haynes), por não haver ficha de tubo com valores; fica dentro do intervalo da fita (Matthey).</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
-        </is>
-      </c>
+      <c r="A52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
+          <t>Legenda</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
+          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.); nas propriedades dependentes da forma, só com valores da forma do dispositivo (regra da forma, v0.8).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+          <t>- Estados da coluna estado:</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
+          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
+          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
+          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
+          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
-        </is>
-      </c>
+      <c r="A63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
+          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
-        </is>
-      </c>
+      <c r="A66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Cuidados</t>
+          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Dentro da janela, típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes. Regista sempre a porosidade e o método de fabrico do estudo.</t>
+          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
-        </is>
-      </c>
+      <c r="A80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
-        </is>
-      </c>
+      <c r="A82" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr"/>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Cuidados</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Níveis de validação</t>
+          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Dentro da janela, típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes. Regista sempre a porosidade e o método de fabrico do estudo.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
+        <is>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Níveis de validação</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
         <is>
           <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
         </is>
@@ -6669,7 +6700,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>típico e mín.: tubo de parede fina recozido 40 % (Alleima 316LVM, coluna "typical", não é mínimo de especificação); máx.: tubo de stent totalmente recozido ~50 % (patente US 6780261 B2, Scimed); valor anterior: 40-60 % (Hanawa T. J Artif Organs 2009;12:73-79); o doi_url é o da patente (fonte do máx.); ficha da Alleima sem URL registado</t>
+          <t>regra da forma: mín. e máx. só com a forma do dispositivo (tubo ou fita; stents cortados a laser de tubo); as duas fontes são de tubo; típico e mín.: tubo de parede fina recozido 40 % (Alleima 316LVM, coluna "typical", não é mínimo de especificação); máx.: tubo de stent totalmente recozido ~50 % (patente US 6780261 B2, Scimed); valor anterior: 40-60 % (Hanawa T. J Artif Organs 2009;12:73-79); o doi_url é o da patente (fonte do máx.); ficha da Alleima sem URL registado</t>
         </is>
       </c>
       <c r="N86" t="n">
@@ -6977,7 +7008,7 @@
         <v>225</v>
       </c>
       <c r="J91" t="n">
-        <v>243</v>
+        <v>225</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -6991,7 +7022,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>Slides: F90 (Co-Cr-W-Ni); Matthey e Haynes 225 GPa; Fort Wayne 243 GPa (https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); típico da chapa (Haynes) por não haver ficha de tubo com valores; a fita (Matthey) dá o intervalo; valor anterior: 243 GPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
+          <t>Slides: F90 (Co-Cr-W-Ni); regra da forma: mín. e máx. só com a forma do dispositivo (tubo ou fita; stents cortados a laser de tubo); valor único nessa forma, ±10 % no Monte Carlo; fita recozida 225 GPa (Matthey); outras formas, só para registo: chapa 225 GPa (Haynes), barra e fio 243 GPa (Fort Wayne, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); intervalo anterior: 225-243 GPa (incluía a barra e o fio); valor anterior: 243 GPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N91" t="n">
@@ -7062,7 +7093,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>intervalo: fita recozida 380-700 MPa (Matthey); típico: chapa solubilizada 476 MPa (Haynes); barra 517 MPa e fio 621 MPa (Fort Wayne, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy) dentro do intervalo; típico da chapa (Haynes) por não haver ficha de tubo com valores; a fita (Matthey) dá o intervalo; valor anterior: 460-500 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
+          <t>regra da forma: mín. e máx. só com a forma do dispositivo (tubo ou fita; stents cortados a laser de tubo); intervalo: fita recozida 380-700 MPa (Matthey); típico: chapa solubilizada 476 MPa (Haynes), por não haver ficha de tubo com valores; outras formas, só para registo: barra 517 MPa e fio 621 MPa (Fort Wayne, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); valor anterior: 460-500 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N92" t="n">
@@ -7119,7 +7150,7 @@
         <v>900</v>
       </c>
       <c r="J93" t="n">
-        <v>1138</v>
+        <v>1000</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -7133,7 +7164,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>fita recozida 900-1000 MPa (Matthey); chapa 996 MPa (Haynes); fio 1138 MPa (Fort Wayne, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); típico da chapa (Haynes) por não haver ficha de tubo com valores; a fita (Matthey) dá o intervalo; valor anterior: 1000-1050 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
+          <t>regra da forma: mín. e máx. só com a forma do dispositivo (tubo ou fita; stents cortados a laser de tubo); intervalo: fita recozida 900-1000 MPa (Matthey); típico: chapa 996 MPa (Haynes), por não haver ficha de tubo com valores; outra forma, só para registo: fio 1138 MPa (Fort Wayne, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); intervalo anterior: 900-1138 MPa (incluía o fio); valor anterior: 1000-1050 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N93" t="n">
@@ -7190,7 +7221,7 @@
         <v>40</v>
       </c>
       <c r="J94" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -7204,7 +7235,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>regra da forma: típico = tubo ou fita (forma dos stents, cortados a laser); o fio só alarga o intervalo; típico e mín.: fita recozida A50mm 40 % (Matthey; a ficha não diz se é valor típico ou mínimo de especificação); máx.: fio recozido 50 % (Fort Wayne, valor típico, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); valor anterior: 50-55 % (Hanawa 2009)</t>
+          <t>regra da forma: mín. e máx. só com a forma do dispositivo (tubo ou fita; stents cortados a laser de tubo); valor único nessa forma, ±10 % no Monte Carlo; fita recozida A50mm 40 % (Matthey; a ficha não diz se é valor típico ou mínimo de especificação); outra forma, só para registo: fio recozido 50 % (Fort Wayne, valor típico, https://fwmetals.com/what-we-do/materials/high-performance-alloys/l-605-alloy); intervalo anterior: 40-50 % (incluía o fio); valor anterior: 50-55 % (Hanawa 2009)</t>
         </is>
       </c>
       <c r="N94" t="n">
@@ -7641,7 +7672,7 @@
         </is>
       </c>
       <c r="I101" t="n">
-        <v>931</v>
+        <v>965</v>
       </c>
       <c r="J101" t="n">
         <v>965</v>
@@ -7658,7 +7689,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>típico e máx.: tubo recozido 140 ksi = 965 MPa (K-Tube; conversão 1 ksi = 6,895 MPa); mín.: fio 931 MPa (Ulbrich, https://www.ulbrich.com/uploads/data-sheets/MP35N-Wire-UNS-R30035.pdf); valor anterior: 930-960 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
+          <t>regra da forma: mín. e máx. só com a forma do dispositivo (tubo ou fita; stents cortados a laser de tubo); valor único nessa forma, ±10 % no Monte Carlo; tubo recozido 140 ksi = 965 MPa (K-Tube; conversão 1 ksi = 6,895 MPa); outra forma, só para registo: fio 931 MPa (Ulbrich, https://www.ulbrich.com/uploads/data-sheets/MP35N-Wire-UNS-R30035.pdf); intervalo anterior: 931-965 MPa (incluía o fio); valor anterior: 930-960 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N101" t="n">
@@ -7715,7 +7746,7 @@
         <v>40</v>
       </c>
       <c r="J102" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="K102" t="inlineStr">
         <is>
@@ -7729,7 +7760,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t>regra da forma: típico = tubo ou fita (forma dos stents, cortados a laser); o fio só alarga o intervalo; típico e mín.: tubo recozido 40 % (K-Tube, tabela "Possible Mechanical Properties": não diz se é típico ou mínimo); máx.: fio recozido 70 % (Ulbrich, valor típico, https://www.ulbrich.com/uploads/data-sheets/MP35N-Wire-UNS-R30035.pdf); valor anterior: 45 % (Hanawa 2009)</t>
+          <t>regra da forma: mín. e máx. só com a forma do dispositivo (tubo ou fita; stents cortados a laser de tubo); valor único nessa forma, ±10 % no Monte Carlo; tubo recozido 40 % (K-Tube, tabela "Possible Mechanical Properties": não diz se é típico ou mínimo); outra forma, só para registo: fio recozido 70 % (Ulbrich, valor típico, https://www.ulbrich.com/uploads/data-sheets/MP35N-Wire-UNS-R30035.pdf); intervalo anterior: 40-70 % (incluía o fio); valor anterior: 45 % (Hanawa 2009)</t>
         </is>
       </c>
       <c r="N102" t="n">
@@ -22115,7 +22146,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.001564</v>
+        <v>0.001689</v>
       </c>
       <c r="C3" t="n">
         <v>0.003111</v>

</xml_diff>

<commit_message>
Cenário P-foco: mapa problema crítico → critérios, peso do problema duplicado; par articular como sensibilidade semiquantitativa
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -16,11 +16,13 @@
     <sheet name="Cenarios" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Tecido" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Parametros" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Problemas_criticos" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materiais'!$A$1:$P$296</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Criterios'!$A$1:$G$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Tecido'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Problemas_criticos'!$A$1:$E$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A90"/>
+  <dimension ref="A1:A96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -470,550 +472,1177 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fonte de verdade: os ficheiros CSV em data/ (materiais, criterios, tecido, cenarios, parametros)</t>
+          <t>Fonte de verdade: os ficheiros CSV em data/ (materiais, criterios, tecido, cenarios, parametros,</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>e este ficheiro (texto da folha LEIA-ME). O base_dados_biomateriais.xlsx é gerado por</t>
+          <t>problemas_criticos)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>e este ficheiro (texto da folha LEIA-ME). O base_dados_biomateriais.xlsx é gerado por</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>scripts/exportar_xlsx.py e não se edita à mão.</t>
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Estado dos valores</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>- Todos os valores são pontos de partida de manuais e revisões e estão marcados "A verificar".</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>- Antes de usar um valor no relatório ou no poster: abre a fonte, confirma o número, preenche a coluna doi_url e muda o estado para "Verificado".</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>- Se a fonte der outro valor, usa o da fonte e regista a página ou tabela na coluna notas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Alterações v0.3 (após revisão crítica)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Densidade deixa de ser proxy de radiopacidade (nova escala de radiopacidade) · σy/E renomeado "proxy material" · Nitinol fora do ranking · K_IC retirado do par articular · "Resistência" retirada da matriz dentária (tração ≠ flexão) · alvos do scaffold passam a cenários · nova folha Cenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Par articular e implante dentário ficam SEMIQUANTITATIVOS (ordinais &gt; 50 % do peso): MCDM quantitativo só para haste, stent (balão) e scaffold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Alterações v0.4 (28 set 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>- Os CSV passam a ser a fonte de verdade; o .xlsx é gerado só com valores (sem fórmulas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>- Novas colunas em materiais.csv: doi_url (a preencher) e valor_texto (propriedades categóricas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>- Nova propriedade "Tipo de expansão" do stent (balão ou autoexpansível), usada na triagem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>- Índices derivados calculados em src/biomat_mcdm/indices.py (σy/E do stent; E_implante/E_osso da haste).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>- Cenários em cenarios.csv; η em parametros.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Alterações v0.5 (1 out 2026): 2.ª ronda do stent</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>- Valores de fichas de fornecedor no 316L (alongamento), no L605 (cedência, módulo, tração) e no MP35N (tração), com o valor anterior na nota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>- L605: o típico é o da chapa (Haynes), por não haver ficha de tubo com valores; a fita (Matthey) dá o intervalo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>- Pt-Cr: cedência com fonte primária (O'Brien 2010, só resumo); módulo, tração e alongamento continuam "A verificar", com fontes secundárias na nota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>- Radiopacidade: rubrica escrita (ver "Rubricas ordinais"), fontes nas 7 linhas e estado "Verificado"; as notas não mudam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>- Densidades do 316L, L605, MP35N e Pt-Cr com fonte. A densidade não é critério do stent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Alterações v0.6 (1 out 2026): 1.ª ronda do scaffold</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>- Rubrica da bioatividade reescrita segundo a classificação de Hench (classes A e B); as notas dos materiais não mudam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>- Regra da porosidade para as propriedades mecânicas dos scaffolds (ver "Cuidados").</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>- 11 linhas do scaffold com fonte primária: porosidade do quitosano/HA, do PLLA e do β-TCP; resistência à compressão da HA; e sete notas ordinais (imprimibilidade, esterilização e bioatividade).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>- A esterilização da HA continua "A verificar".</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Alterações v0.7 (1 out 2026): 2.ª ronda do scaffold</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>- Regra do típico: típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>- β-TCP: resistência 0,35-7,72 MPa, típico 2. PCL/β-TCP: porosidade típica 70 % (especificação dos scaffolds por FDM).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>- HA: tempo de degradação tratado como não reabsorvível (mínimo 42 meses; máximo e típico = pior valor observado nos outros materiais, como a opção O2 do stent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>- PLLA definido como scaffold impresso; degradação 24-60 meses, com dados de PLLA maciço.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>- Vidro 45S5: resistência 0,2-1,1 MPa e degradação 6-24 meses (dados de partículas). O módulo fica sem fonte primária.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>- Quitosano/HA: módulo e resistência cerca de dez vezes abaixo dos valores anteriores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>- Porosidades do PCL, do PLGA e da HA com fonte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Alterações v0.8 (2 out 2026): regra da forma revista (stent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>- Regra da forma: nas propriedades dependentes da forma do produto, min, max e tipico cobrem só a forma usada no dispositivo (no stent: tubo ou fita); os valores de outras formas (fio, barra, chapa) ficam só na coluna notas. Se a forma do dispositivo tiver um único valor, min = max e o Monte Carlo aplica ±10 % (incerteza_valor_unico em parametros.csv).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>- Linhas revistas: L605 módulo 225 (antes 225-243), tração 900-1000 (antes 900-1138), alongamento 40 (antes 40-50); MP35N tração 965 (antes 931-965), alongamento 40 (antes 40-70). Sem alteração: 316L alongamento 40-50 e L605 cedência 380-700. Os típicos não mudaram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>- Exceção mantida no L605: o típico da cedência e da tração é o da chapa (Haynes), por não haver ficha de tubo com valores; fica dentro do intervalo da fita (Matthey).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Alterações v0.9 (3 out 2026): problemas críticos do professor</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>- Novo problemas_criticos.csv: para cada caso, os critérios que respondem ao problema crítico indicado pelo professor (2 out 2026), com ligação direta ou indireta e justificação. Folha Problemas_criticos no .xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>- Novo parâmetro fator_foco_problema = 2 (valor de desenho) e novo cenário P-foco: peso dos critérios de ligação direta x2, restantes renormalizados; sensibilidade com direta + indireta; no par articular, só como sensibilidade semiquantitativa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>- Implante dentário: a corrosão ainda não é critério (a acrescentar).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Legenda</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.); nas propriedades dependentes da forma, só com valores da forma do dispositivo (regra da forma, v0.8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>- Estados da coluna estado:</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Cuidados</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Dentro da janela, típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes. Regista sempre a porosidade e o método de fabrico do estudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Níveis de validação</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="53" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>caso_componente</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>problema</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>criterio</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>ligacao</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>justificacao</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Prótese da anca | Par articular</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Desgaste e libertação de partículas</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Taxa de desgaste linear</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Partículas de desgaste do polietileno: osteólise e descolamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Prótese da anca | Par articular</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Desgaste e libertação de partículas</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Segurança iónica / risco ALTR (ordinal 1-5)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Iões e partículas metálicas; também critério de triagem (≥ 2, exclui o MoM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Prótese da anca | Par articular</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Desgaste e libertação de partículas</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Compatibilidade galvânica cabeça-cone (ordinal 1-5)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Corrosão por fretting na junção cabeça-cone liberta iões e partículas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Prótese da anca | Par articular</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Desgaste e libertação de partículas</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Dureza da cabeça</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>indireta</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Riscos por terceiro corpo aceleram o desgaste do contraface</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Prótese da anca | Par articular</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Desgaste e libertação de partículas</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>indireta</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A oxidação do polietileno irradiado acelera o desgaste</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Prótese da anca | Haste femoral</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Desgaste e libertação de partículas</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Resistência à corrosão (ordinal 1-5)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Libertação iónica da haste</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Implante dentário</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Integração com o osso</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Evidência clínica de osteointegração (ordinal 1-5)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Função principal do implante</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Estado dos valores</t>
+          <t>Implante dentário</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Integração com o osso</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Módulo de Young</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>indireta</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Transferência de carga ao osso e perda óssea marginal</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>- Todos os valores são pontos de partida de manuais e revisões e estão marcados "A verificar".</t>
+          <t>Stent vascular</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Resistência mecânica</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Índice material de recuo elástico σy/E (proxy)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Recuo elástico depois da expansão</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- Antes de usar um valor no relatório ou no poster: abre a fonte, confirma o número, preenche a coluna doi_url e muda o estado para "Verificado".</t>
+          <t>Stent vascular</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Resistência mecânica</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Alongamento na rotura</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Expansão sem fratura</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>- Se a fonte der outro valor, usa o da fonte e regista a página ou tabela na coluna notas.</t>
+          <t>Stent vascular</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Resistência mecânica</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Resistência à tração</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Resistência radial e fadiga pulsátil</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Stent vascular</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Resistência mecânica</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Módulo de Young</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Rigidez radial com struts finos</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Alterações v0.3 (após revisão crítica)</t>
+          <t>Stent vascular</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Biocompatibilidade</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Espessura típica de strut</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Struts finos: menos reestenose e trombose (propriedade do dispositivo)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Densidade deixa de ser proxy de radiopacidade (nova escala de radiopacidade) · σy/E renomeado "proxy material" · Nitinol fora do ranking · K_IC retirado do par articular · "Resistência" retirada da matriz dentária (tração ≠ flexão) · alvos do scaffold passam a cenários · nova folha Cenarios</t>
+          <t>Stent vascular</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Biocompatibilidade</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Tempo de reabsorção (só cenário B)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>indireta</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Presença permanente vs reabsorção; só no cenário B</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Suporte celular</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Porosidade</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Poros interligados para adesão, migração e vascularização</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Par articular e implante dentário ficam SEMIQUANTITATIVOS (ordinais &gt; 50 % do peso): MCDM quantitativo só para haste, stent (balão) e scaffold.</t>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Suporte celular</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Bioatividade (ordinal 1-5)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Osteocondução e ligação ao osso</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Degradação controlada</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Tempo de degradação</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>direta</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Acompanhar a formação de osso novo</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Alterações v0.4 (28 set 2026)</t>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Suporte celular</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Imprimibilidade 3D (ordinal 1-5)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>indireta</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Controlo da arquitetura dos poros</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>- Os CSV passam a ser a fonte de verdade; o .xlsx é gerado só com valores (sem fórmulas).</t>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Suporte celular</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Resistência à compressão (scaffold)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>indireta</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Suporte mecânico enquanto o osso se forma (leitura ampla)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>- Novas colunas em materiais.csv: doi_url (a preencher) e valor_texto (propriedades categóricas).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>- Nova propriedade "Tipo de expansão" do stent (balão ou autoexpansível), usada na triagem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>- Índices derivados calculados em src/biomat_mcdm/indices.py (σy/E do stent; E_implante/E_osso da haste).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>- Cenários em cenarios.csv; η em parametros.csv.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Alterações v0.5 (1 out 2026): 2.ª ronda do stent</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>- Valores de fichas de fornecedor no 316L (alongamento), no L605 (cedência, módulo, tração) e no MP35N (tração), com o valor anterior na nota.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>- L605: o típico é o da chapa (Haynes), por não haver ficha de tubo com valores; a fita (Matthey) dá o intervalo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>- Pt-Cr: cedência com fonte primária (O'Brien 2010, só resumo); módulo, tração e alongamento continuam "A verificar", com fontes secundárias na nota.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>- Radiopacidade: rubrica escrita (ver "Rubricas ordinais"), fontes nas 7 linhas e estado "Verificado"; as notas não mudam.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>- Densidades do 316L, L605, MP35N e Pt-Cr com fonte. A densidade não é critério do stent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Alterações v0.6 (1 out 2026): 1.ª ronda do scaffold</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>- Rubrica da bioatividade reescrita segundo a classificação de Hench (classes A e B); as notas dos materiais não mudam.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>- Regra da porosidade para as propriedades mecânicas dos scaffolds (ver "Cuidados").</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>- 11 linhas do scaffold com fonte primária: porosidade do quitosano/HA, do PLLA e do β-TCP; resistência à compressão da HA; e sete notas ordinais (imprimibilidade, esterilização e bioatividade).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>- A esterilização da HA continua "A verificar".</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Alterações v0.7 (1 out 2026): 2.ª ronda do scaffold</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>- Regra do típico: típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>- β-TCP: resistência 0,35-7,72 MPa, típico 2. PCL/β-TCP: porosidade típica 70 % (especificação dos scaffolds por FDM).</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>- HA: tempo de degradação tratado como não reabsorvível (mínimo 42 meses; máximo e típico = pior valor observado nos outros materiais, como a opção O2 do stent).</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>- PLLA definido como scaffold impresso; degradação 24-60 meses, com dados de PLLA maciço.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>- Vidro 45S5: resistência 0,2-1,1 MPa e degradação 6-24 meses (dados de partículas). O módulo fica sem fonte primária.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>- Quitosano/HA: módulo e resistência cerca de dez vezes abaixo dos valores anteriores.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>- Porosidades do PCL, do PLGA e da HA com fonte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Alterações v0.8 (2 out 2026): regra da forma revista (stent)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>- Regra da forma: nas propriedades dependentes da forma do produto, min, max e tipico cobrem só a forma usada no dispositivo (no stent: tubo ou fita); os valores de outras formas (fio, barra, chapa) ficam só na coluna notas. Se a forma do dispositivo tiver um único valor, min = max e o Monte Carlo aplica ±10 % (incerteza_valor_unico em parametros.csv).</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>- Linhas revistas: L605 módulo 225 (antes 225-243), tração 900-1000 (antes 900-1138), alongamento 40 (antes 40-50); MP35N tração 965 (antes 931-965), alongamento 40 (antes 40-70). Sem alteração: 316L alongamento 40-50 e L605 cedência 380-700. Os típicos não mudaram.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>- Exceção mantida no L605: o típico da cedência e da tração é o da chapa (Haynes), por não haver ficha de tubo com valores; fica dentro do intervalo da fita (Matthey).</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Legenda</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.); nas propriedades dependentes da forma, só com valores da forma do dispositivo (regra da forma, v0.8).</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>- Estados da coluna estado:</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Cuidados</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Dentro da janela, típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes. Regista sempre a porosidade e o método de fabrico do estudo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>Níveis de validação</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Suporte celular</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Módulo de compressão (scaffold)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>indireta</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Suporte mecânico enquanto o osso se forma (leitura ampla)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22432,7 +23061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -22656,6 +23285,23 @@
         </is>
       </c>
       <c r="C13" t="inlineStr">
+        <is>
+          <t>Todos os quantitativos</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P-foco</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Foco no problema crítico do professor (2 out 2026): peso dos critérios de ligação direta x2 (fator_foco_problema), restantes renormalizados; sensibilidade: direta + indireta (data/problemas_criticos.csv). Par articular: sensibilidade semiquantitativa à parte</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>Todos os quantitativos</t>
         </is>
@@ -23018,7 +23664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -23073,6 +23719,21 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fator_foco_problema</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cenário P-foco: o peso dos critérios ligados ao problema crítico do professor (2 out 2026; data/problemas_criticos.csv) é multiplicado por este fator e os pesos são renormalizados; valor de desenho</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Implante dentário: critério de corrosão, osteointegração com fontes e análise semiquantitativa com P-foco
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -19,10 +19,10 @@
     <sheet name="Problemas_criticos" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materiais'!$A$1:$P$296</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Materiais'!$A$1:$P$301</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Criterios'!$A$1:$G$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Tecido'!$A$1:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Problemas_criticos'!$A$1:$E$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Problemas_criticos'!$A$1:$E$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A96"/>
+  <dimension ref="A1:A104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -800,7 +800,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>- Implante dentário: a corrosão ainda não é critério (a acrescentar).</t>
+          <t>- Implante dentário: a corrosão passa a critério na v0.10.</t>
         </is>
       </c>
     </row>
@@ -810,229 +810,233 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Legenda</t>
+          <t>Alterações v0.10 (3 out 2026): implante dentário centrado na osteointegração e na corrosão</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.); nas propriedades dependentes da forma, só com valores da forma do dispositivo (regra da forma, v0.8).</t>
+          <t>- Novo critério "Resistência à corrosão em meio oral (ordinal 1-5)", de benefício, peso 0,15 (problema crítico do docente); para lhe dar peso: estética 0,15 → 0,10, módulo 0,20 → 0,15 e a densidade deixa de ser critério do dentário (a propriedade fica na base).</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
+          <t>- Corrosão: Ti grau 4 = 3, Ti-6Al-4V ELI = 3, Ti-Zr = 3 (4 como sensibilidade), Y-TZP = 4, PEEK = 5.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>- Estados da coluna estado:</t>
+          <t>- Osteointegração com fontes e rubrica nova; Ti-6Al-4V ELI 4 → 2 (sem estudos clínicos dedicados no corpo do implante dentário).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
+          <t>- Estado "Verificado" com a nota "só resumo; nota segundo a rubrica do leia_me" (decisão do André).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
+          <t>- Peso ordinal do dentário: 0,70 (antes 0,60); o caso continua SEMIQUANTITATIVO: ranking e P-foco só como indicação (results/semiquantitativos.csv).</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
-        </is>
-      </c>
+      <c r="A65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+          <t>Legenda</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.); nas propriedades dependentes da forma, só com valores da forma do dispositivo (regra da forma, v0.8).</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
+          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>- Estados da coluna estado:</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
+          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
+          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
+          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
+          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>- Osteointegração: 5 = padrão-ouro com décadas de dados; 3 = dados clínicos a médio prazo; 1 = bioinerte com fraca aposição óssea</t>
-        </is>
-      </c>
+      <c r="A76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
+          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
-        </is>
-      </c>
+      <c r="A79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+          <t>- Osteointegração (implante dentário; revista a 3 out 2026, pelo tipo e duração da evidência clínica do corpo do implante): 5 = coortes com 10 anos ou mais e milhares de implantes, mais meta-análises a 10 anos; 4 = ensaios aleatorizados ou meta-análises com centenas de implantes e pelo menos um estudo a 10 anos; 3 = meta-análises a 1-5 anos ou coortes de 10 anos pequenas e heterogéneas; 2 = uso clínico sem estudos clínicos dedicados (só equivalência em estudos animais); 1 = só evidência pré-clínica. Fontes por material na coluna referencia e em NOTAS_METODOLOGICAS.md.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
+          <t>- Corrosão em meio oral (implante dentário, 3 out 2026): 5 = inerte em meio oral (sem corrosão eletroquímica nem degradação com efeito documentado); 4 = sem corrosão eletroquímica, mas com degradação lenta documentada em meio húmido ou oral (envelhecimento, absorção de água); 3 = metal passivo estável em saliva, atacado só em condições agressivas (fluoreto em meio ácido, tribocorrosão), com libertação de iões ou partículas documentada; 2 = metal atacado em condições orais comuns ou com acoplamento galvânico relevante; 1 = sem filme protetor estável.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Cuidados</t>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Dentro da janela, típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes. Regista sempre a porosidade e o método de fabrico do estudo.</t>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
         </is>
       </c>
     </row>
@@ -1042,12 +1046,60 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
+          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Cuidados</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Dentro da janela, típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes. Regista sempre a porosidade e o método de fabrico do estudo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
           <t>Níveis de validação</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
+    <row r="104">
+      <c r="A104" t="inlineStr">
         <is>
           <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
         </is>
@@ -1064,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1320,17 +1372,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Stent vascular</t>
+          <t>Implante dentário</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Resistência mecânica</t>
+          <t>Corrosão</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Índice material de recuo elástico σy/E (proxy)</t>
+          <t>Resistência à corrosão em meio oral (ordinal 1-5)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1340,7 +1392,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Recuo elástico depois da expansão</t>
+          <t>Critério acrescentado para o problema crítico</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1409,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Alongamento na rotura</t>
+          <t>Índice material de recuo elástico σy/E (proxy)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1367,7 +1419,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Expansão sem fratura</t>
+          <t>Recuo elástico depois da expansão</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1436,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Resistência à tração</t>
+          <t>Alongamento na rotura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1394,7 +1446,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Resistência radial e fadiga pulsátil</t>
+          <t>Expansão sem fratura</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1463,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Módulo de Young</t>
+          <t>Resistência à tração</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1421,7 +1473,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Rigidez radial com struts finos</t>
+          <t>Resistência radial e fadiga pulsátil</t>
         </is>
       </c>
     </row>
@@ -1433,12 +1485,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Biocompatibilidade</t>
+          <t>Resistência mecânica</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Espessura típica de strut</t>
+          <t>Módulo de Young</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1448,7 +1500,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Struts finos: menos reestenose e trombose (propriedade do dispositivo)</t>
+          <t>Rigidez radial com struts finos</t>
         </is>
       </c>
     </row>
@@ -1465,44 +1517,44 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tempo de reabsorção (só cenário B)</t>
+          <t>Espessura típica de strut</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>indireta</t>
+          <t>direta</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Presença permanente vs reabsorção; só no cenário B</t>
+          <t>Struts finos: menos reestenose e trombose (propriedade do dispositivo)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Suporte celular</t>
+          <t>Biocompatibilidade</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Porosidade</t>
+          <t>Tempo de reabsorção (só cenário B)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>direta</t>
+          <t>indireta</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Poros interligados para adesão, migração e vascularização</t>
+          <t>Presença permanente vs reabsorção; só no cenário B</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1571,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Bioatividade (ordinal 1-5)</t>
+          <t>Porosidade</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1529,7 +1581,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Osteocondução e ligação ao osso</t>
+          <t>Poros interligados para adesão, migração e vascularização</t>
         </is>
       </c>
     </row>
@@ -1541,12 +1593,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Degradação controlada</t>
+          <t>Suporte celular</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tempo de degradação</t>
+          <t>Bioatividade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1556,7 +1608,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Acompanhar a formação de osso novo</t>
+          <t>Osteocondução e ligação ao osso</t>
         </is>
       </c>
     </row>
@@ -1568,22 +1620,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Suporte celular</t>
+          <t>Degradação controlada</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Imprimibilidade 3D (ordinal 1-5)</t>
+          <t>Tempo de degradação</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>indireta</t>
+          <t>direta</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Controlo da arquitetura dos poros</t>
+          <t>Acompanhar a formação de osso novo</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1652,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Resistência à compressão (scaffold)</t>
+          <t>Imprimibilidade 3D (ordinal 1-5)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1610,7 +1662,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Suporte mecânico enquanto o osso se forma (leitura ampla)</t>
+          <t>Controlo da arquitetura dos poros</t>
         </is>
       </c>
     </row>
@@ -1627,22 +1679,49 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>Resistência à compressão (scaffold)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>indireta</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Suporte mecânico enquanto o osso se forma (leitura ampla)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Suporte celular</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>Módulo de compressão (scaffold)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>indireta</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Suporte mecânico enquanto o osso se forma (leitura ampla)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E21"/>
+  <autoFilter ref="A1:E22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1653,7 +1732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P296"/>
+  <dimension ref="A1:P301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5596,7 +5675,17 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
+          <t>Adell R et al. Int J Oral Maxillofac Implants 1990;5:347-359 (PMID 2094653); Howe MS et al. J Dent 2019;84:9-21</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jdent.2019.03.008</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>só resumo; nota segundo a rubrica do leia_me; Adell 1990: 4636 implantes de Ti cp (grau não indicado no resumo), sobrevivência 86 % (mandíbula) e 78 % (maxila) aos 15 anos; Howe 2019: meta-análise, 96,4 % aos 10 anos (sistemas contemporâneos, sem separar por material); Müller F et al. Clin Oral Implants Res 2024;35:77-88 (https://doi.org/10.1111/clr.14199): braço de Ti grau IV 95,8 % aos 10 anos; valor anterior: 5</t>
         </is>
       </c>
       <c r="N58" t="n">
@@ -5604,7 +5693,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -5955,22 +6044,32 @@
         </is>
       </c>
       <c r="I64" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J64" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
+          <t>Shah FA et al. Mater Sci Eng C 2016;62:960-966; Johansson CB et al. Int J Oral Maxillofac Implants 1998;13:315-321 (PMID 9638001)</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.msec.2016.01.032</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>só resumo; nota segundo a rubrica do leia_me; sem séries clínicas que identifiquem a liga no corpo do implante dentário; Shah 2016 (revisão): não existem estudos clínicos comparativos com o Ti cp; Johansson 1998 (coelho): torque de remoção menor do que o do Ti cp; valor anterior: 4</t>
         </is>
       </c>
       <c r="N64" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -6328,7 +6427,17 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
+          <t>Müller F et al. Clin Oral Implants Res 2024;35:77-88; Altuna P et al. Int J Oral Maxillofac Surg 2016;45:842-850</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/clr.14199</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>só resumo; nota segundo a rubrica do leia_me; Müller 2024: ensaio aleatorizado em boca dividida, TiZr 98,9 % vs Ti grau IV 95,8 % aos 10 anos (36 doentes na análise ITT); Altuna 2016 (https://doi.org/10.1016/j.ijom.2016.01.004): 922 implantes, 97,7 % aos 2 anos; ensaio patrocinado pela Institut Straumann AG (Müller 2015, BMC Oral Health 15:123, texto completo); valor anterior: 4</t>
         </is>
       </c>
       <c r="N70" t="n">
@@ -6336,7 +6445,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -6704,7 +6813,17 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
+          <t>Pieralli S et al. J Dent Res 2017;96:38-46; Roehling S et al. Clin Oral Implants Res 2018;29(S16):135-153</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/0022034516664043</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>só resumo; nota segundo a rubrica do leia_me; Pieralli 2017: 398 implantes, 95,6 % aos 12 meses; Roehling 2018 (https://doi.org/10.1111/clr.13352): 98,3 % (1 ano), 97,2 % (2 anos); Roehling 2026 (https://doi.org/10.1111/clr.70089): 97,7 % aos 10 anos, 35 implantes, financiado pela Straumann; outros sistemas 62-80 % (Herber 2025, https://doi.org/10.1186/s40729-025-00655-1; Steyer 2021, https://doi.org/10.3390/ma14226738); consenso ITI 2018 (Morton, https://doi.org/10.1111/clr.13298): preferir implantes de uma peça; valor anterior: 3</t>
         </is>
       </c>
       <c r="N76" t="n">
@@ -6712,7 +6831,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -7070,7 +7189,17 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Escala ordinal definida no trabalho (rubrica em LEIA-ME): justificar com literatura</t>
+          <t>Najeeb S et al. J Oral Implantol 2016;42:512-516; Mishra S, Chowdhary R. Clin Implant Dent Relat Res 2019;21:208-222</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1563/aaid-joi-d-16-00072</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>só resumo; nota segundo a rubrica do leia_me; só evidência pré-clínica; nos estudos animais o PEEK sem revestimento foi menos osteogénico do que o titânio (Najeeb 2016); faltam ensaios clínicos (Mishra 2019, https://doi.org/10.1111/cid.12706); valor anterior: 1</t>
         </is>
       </c>
       <c r="N82" t="n">
@@ -7078,7 +7207,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -17354,22 +17483,22 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Stent vascular</t>
+          <t>Implante dentário</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Estrutura do stent</t>
+          <t>Corpo do implante</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Aço inox 316L</t>
+          <t>Ti cp grau 4</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>ASTM F138</t>
+          <t>ASTM F67</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -17379,12 +17508,12 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Clínico (1.ª geração)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>Compatibilidade com RM (ordinal 1-5)</t>
+          <t>Resistência à corrosão em meio oral (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -17393,49 +17522,54 @@
         </is>
       </c>
       <c r="I240" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J240" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K240" t="inlineStr">
         <is>
-          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
+          <t>Nakagawa M et al. J Dent Res 1999;78:1568-1572; Apaza-Bedoya K et al. J Periodontal Res 2017;52:946-954</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/00220345990780091201</t>
         </is>
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t>MR-condicional; artefacto maior</t>
+          <t>só resumo; nota segundo a rubrica do leia_me; filme passivo destruído com HF acima de cerca de 30 ppm (Nakagawa 1999; limiar de pH e fluoreto no texto completo, não lido); tribocorrosão na ligação implante-pilar (Apaza-Bedoya 2017, https://doi.org/10.1111/jre.12469); mais Ti na placa com peri-implantite (Safioti 2017, https://doi.org/10.1902/jop.2016.160524), sem causalidade provada (Mombelli 2018, https://doi.org/10.1111/clr.13305)</t>
         </is>
       </c>
       <c r="N240" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Stent vascular</t>
+          <t>Implante dentário</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Estrutura do stent</t>
+          <t>Corpo do implante</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Co-Cr L605</t>
+          <t>Ti-6Al-4V ELI</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>ASTM F90</t>
+          <t>ASTM F136</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -17450,7 +17584,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>Compatibilidade com RM (ordinal 1-5)</t>
+          <t>Resistência à corrosão em meio oral (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -17466,12 +17600,17 @@
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
+          <t>Nakagawa M et al. Dent Mater J 2001;20:305-314; Huang HH. Biomaterials 2003;24:275-282</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.4012/dmj.20.305</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>MR-condicional</t>
+          <t>só resumo; nota segundo a rubrica do leia_me; também atacada por fluoreto em meio ácido, sem diferença face ao Ti cp indicada no resumo (Nakagawa 2001); filme destruído com NaF acima de 0,1 % em saliva artificial a pH 5 (Huang 2003, https://doi.org/10.1016/s0142-9612(02)00315-0); a libertação de Al e V é questão de biocompatibilidade e não entra nesta nota</t>
         </is>
       </c>
       <c r="N241" t="n">
@@ -17479,29 +17618,29 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Stent vascular</t>
+          <t>Implante dentário</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Estrutura do stent</t>
+          <t>Corpo do implante</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Co-Ni-Cr-Mo MP35N</t>
+          <t>Ti-Zr (~15% Zr)</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>ASTM F562</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
@@ -17516,7 +17655,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>Compatibilidade com RM (ordinal 1-5)</t>
+          <t>Resistência à corrosão em meio oral (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -17532,12 +17671,17 @@
       </c>
       <c r="K242" t="inlineStr">
         <is>
-          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
+          <t>Akimoto T et al. J Biomed Mater Res B 2018;106:73-79; Grandin HM, Berner S, Dard M. Materials 2012;5:1348-1360</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/jbm.b.33811</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>MR-condicional</t>
+          <t>só resumo; nota segundo a rubrica do leia_me; in vitro igual ou melhor do que o Ti cp, mas com composições diferentes da do Roxolid (Akimoto 2018: Ti-30Zr em % mol; Santos 2023, https://doi.org/10.3390/ma16051826: Ti-15Zr em PBS); Grandin 2012 (https://doi.org/10.3390/ma5081348, texto completo): corrosão pelo menos tão boa como a do Ti puro, autores da Straumann; sem dados com fluoreto; 4 só como cenário de sensibilidade</t>
         </is>
       </c>
       <c r="N242" t="n">
@@ -17545,34 +17689,34 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Stent vascular</t>
+          <t>Implante dentário</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Estrutura do stent</t>
+          <t>Corpo do implante</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Pt-Cr</t>
+          <t>Zircónia Y-TZP</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ISO 13356</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Cerâmico</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -17582,7 +17726,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>Compatibilidade com RM (ordinal 1-5)</t>
+          <t>Resistência à corrosão em meio oral (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -17591,64 +17735,69 @@
         </is>
       </c>
       <c r="I243" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J243" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K243" t="inlineStr">
         <is>
-          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
+          <t>Chevalier J et al. J Am Ceram Soc 2009;92:1901-1920; Kocjan A et al. Dent Mater 2021;37:443-453</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/j.1551-2916.2009.03278.x</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>Pt paramagnético</t>
+          <t>só resumo; nota segundo a rubrica do leia_me; sem corrosão eletroquímica; degradação a baixa temperatura em meio húmido (Chevalier 2009); in vivo na boca, fração monoclínica cerca de 8 % aos 6 meses e 12 % aos 24 meses (Kocjan 2021, https://doi.org/10.1016/j.dental.2020.11.023)</t>
         </is>
       </c>
       <c r="N243" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Stent vascular</t>
+          <t>Implante dentário</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Estrutura do stent</t>
+          <t>Corpo do implante</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Nitinol (autoexpansível)</t>
+          <t>PEEK</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>ASTM F2063</t>
+          <t>ASTM F2026</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Metal (superelástico)</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>Excluído (autoexpansível: só discussão)</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>Compatibilidade com RM (ordinal 1-5)</t>
+          <t>Resistência à corrosão em meio oral (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
@@ -17657,27 +17806,32 @@
         </is>
       </c>
       <c r="I244" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J244" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
+          <t>Kurtz SM, Devine JN. Biomaterials 2007;28:4845-4869; Liebermann A et al. J Prosthet Dent 2016;115:321-328</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.biomaterials.2007.07.013</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>MR-condicional</t>
+          <t>só resumo; nota segundo a rubrica do leia_me; não hidrolisa, absorção de água cerca de 0,5 % (Kurtz e Devine 2007, texto completo, secção de resistência química); menor absorção e solubilidade em saliva entre polímeros CAD/CAM (Liebermann 2016, https://doi.org/10.1016/j.prosdent.2015.09.004)</t>
         </is>
       </c>
       <c r="N244" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -17694,22 +17848,22 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Liga de Mg WE43 (bioabsorvível)</t>
+          <t>Aço inox 316L</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F138</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>Metal biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>Clínico (Magmaris)</t>
+          <t>Clínico (1.ª geração)</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -17723,10 +17877,10 @@
         </is>
       </c>
       <c r="I245" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J245" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K245" t="inlineStr">
         <is>
@@ -17735,11 +17889,11 @@
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>Artefacto mínimo</t>
+          <t>MR-condicional; artefacto maior</t>
         </is>
       </c>
       <c r="N245" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O245" t="inlineStr">
         <is>
@@ -17760,22 +17914,22 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>PLLA (bioabsorvível)</t>
+          <t>Co-Cr L605</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F90</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Polímero biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>Descontinuado (Absorb, 2017)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -17789,10 +17943,10 @@
         </is>
       </c>
       <c r="I246" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J246" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K246" t="inlineStr">
         <is>
@@ -17801,11 +17955,11 @@
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>Polímero; marcadores metálicos nas extremidades</t>
+          <t>MR-condicional</t>
         </is>
       </c>
       <c r="N246" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O246" t="inlineStr">
         <is>
@@ -17826,12 +17980,12 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Aço inox 316L</t>
+          <t>Co-Ni-Cr-Mo MP35N</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>ASTM F138</t>
+          <t>ASTM F562</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
@@ -17841,12 +17995,12 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Clínico (1.ª geração)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>Radiopacidade (ordinal 1-5)</t>
+          <t>Compatibilidade com RM (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -17862,17 +18016,12 @@
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
-        </is>
-      </c>
-      <c r="L247" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1186/1745-6215-11-1</t>
+          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
         </is>
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>Visibilidade reduzida com struts finos; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
+          <t>MR-condicional</t>
         </is>
       </c>
       <c r="N247" t="n">
@@ -17880,7 +18029,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -17897,12 +18046,12 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Co-Cr L605</t>
+          <t>Pt-Cr</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>ASTM F90</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
@@ -17917,7 +18066,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>Radiopacidade (ordinal 1-5)</t>
+          <t>Compatibilidade com RM (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -17926,32 +18075,27 @@
         </is>
       </c>
       <c r="I248" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J248" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
-        </is>
-      </c>
-      <c r="L248" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1186/1745-6215-11-1</t>
+          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>W na liga aumenta a radiopacidade; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
+          <t>Pt paramagnético</t>
         </is>
       </c>
       <c r="N248" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -17968,27 +18112,27 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Co-Ni-Cr-Mo MP35N</t>
+          <t>Nitinol (autoexpansível)</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>ASTM F562</t>
+          <t>ASTM F2063</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Metal (superelástico)</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Excluído (autoexpansível: só discussão)</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>Radiopacidade (ordinal 1-5)</t>
+          <t>Compatibilidade com RM (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -17997,32 +18141,27 @@
         </is>
       </c>
       <c r="I249" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J249" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
-        </is>
-      </c>
-      <c r="L249" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1186/1745-6215-11-1</t>
+          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
         </is>
       </c>
       <c r="M249" t="inlineStr">
         <is>
-          <t>ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
+          <t>MR-condicional</t>
         </is>
       </c>
       <c r="N249" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -18039,7 +18178,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Pt-Cr</t>
+          <t>Liga de Mg WE43 (bioabsorvível)</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -18049,17 +18188,17 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Metal biodegradável</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Clínico (Magmaris)</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>Radiopacidade (ordinal 1-5)</t>
+          <t>Compatibilidade com RM (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
@@ -18075,17 +18214,12 @@
       </c>
       <c r="K250" t="inlineStr">
         <is>
-          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
-        </is>
-      </c>
-      <c r="L250" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1186/1745-6215-11-1</t>
+          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
         </is>
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>Pt: número atómico elevado; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
+          <t>Artefacto mínimo</t>
         </is>
       </c>
       <c r="N250" t="n">
@@ -18093,7 +18227,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -18110,27 +18244,27 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Nitinol (autoexpansível)</t>
+          <t>PLLA (bioabsorvível)</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>ASTM F2063</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Metal (superelástico)</t>
+          <t>Polímero biodegradável</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Excluído (autoexpansível: só discussão)</t>
+          <t>Descontinuado (Absorb, 2017)</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>Radiopacidade (ordinal 1-5)</t>
+          <t>Compatibilidade com RM (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
@@ -18139,32 +18273,27 @@
         </is>
       </c>
       <c r="I251" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J251" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K251" t="inlineStr">
         <is>
-          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
-        </is>
-      </c>
-      <c r="L251" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1186/1745-6215-11-1</t>
+          <t>Shellock FG / MRIsafety.com; ASTM F2182 (aquecimento) e F2119 (artefactos): confirmar</t>
         </is>
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>Precisa de marcadores; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
+          <t>Polímero; marcadores metálicos nas extremidades</t>
         </is>
       </c>
       <c r="N251" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -18181,22 +18310,22 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Liga de Mg WE43 (bioabsorvível)</t>
+          <t>Aço inox 316L</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F138</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Metal biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Clínico (Magmaris)</t>
+          <t>Clínico (1.ª geração)</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -18210,10 +18339,10 @@
         </is>
       </c>
       <c r="I252" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J252" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K252" t="inlineStr">
         <is>
@@ -18227,11 +18356,11 @@
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>Precisa de marcadores radiopacos; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
+          <t>Visibilidade reduzida com struts finos; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N252" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O252" t="inlineStr">
         <is>
@@ -18252,22 +18381,22 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>PLLA (bioabsorvível)</t>
+          <t>Co-Cr L605</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F90</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Polímero biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Descontinuado (Absorb, 2017)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -18281,10 +18410,10 @@
         </is>
       </c>
       <c r="I253" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J253" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K253" t="inlineStr">
         <is>
@@ -18298,11 +18427,11 @@
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>Marcadores de Pt nas extremidades; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
+          <t>W na liga aumenta a radiopacidade; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N253" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O253" t="inlineStr">
         <is>
@@ -18323,12 +18452,12 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Aço inox 316L</t>
+          <t>Co-Ni-Cr-Mo MP35N</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>ASTM F138</t>
+          <t>ASTM F562</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -18338,12 +18467,12 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Clínico (1.ª geração)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Radiopacidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
@@ -18352,27 +18481,32 @@
         </is>
       </c>
       <c r="I254" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J254" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K254" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>Stent farmacológico → EtO (o fármaco limita)</t>
+          <t>ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N254" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -18389,12 +18523,12 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Co-Cr L605</t>
+          <t>Pt-Cr</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>ASTM F90</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -18409,7 +18543,7 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Radiopacidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
@@ -18418,27 +18552,32 @@
         </is>
       </c>
       <c r="I255" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J255" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K255" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>Idem</t>
+          <t>Pt: número atómico elevado; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N255" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -18455,27 +18594,27 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Co-Ni-Cr-Mo MP35N</t>
+          <t>Nitinol (autoexpansível)</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>ASTM F562</t>
+          <t>ASTM F2063</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Metal (superelástico)</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Excluído (autoexpansível: só discussão)</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Radiopacidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
@@ -18484,27 +18623,32 @@
         </is>
       </c>
       <c r="I256" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J256" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K256" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>Idem</t>
+          <t>Precisa de marcadores; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N256" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -18521,7 +18665,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Pt-Cr</t>
+          <t>Liga de Mg WE43 (bioabsorvível)</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -18531,17 +18675,17 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Metal biodegradável</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Clínico (Magmaris)</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Radiopacidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -18550,27 +18694,32 @@
         </is>
       </c>
       <c r="I257" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J257" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K257" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M257" t="inlineStr">
         <is>
-          <t>Idem</t>
+          <t>Precisa de marcadores radiopacos; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N257" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -18587,27 +18736,27 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Nitinol (autoexpansível)</t>
+          <t>PLLA (bioabsorvível)</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>ASTM F2063</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Metal (superelástico)</t>
+          <t>Polímero biodegradável</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Excluído (autoexpansível: só discussão)</t>
+          <t>Descontinuado (Absorb, 2017)</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Radiopacidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -18616,27 +18765,32 @@
         </is>
       </c>
       <c r="I258" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J258" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K258" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Allocco DJ et al. Trials 2010;11:1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr); rubrica no LEIA-ME (teor de elementos de Z alto)</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/1745-6215-11-1</t>
         </is>
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>Sem revestimento de fármaco (periférico)</t>
+          <t>Marcadores de Pt nas extremidades; ordem suportada por Allocco 2010 (densidade como comparação direta); notas segundo a rubrica do leia_me</t>
         </is>
       </c>
       <c r="N258" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -18653,22 +18807,22 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Liga de Mg WE43 (bioabsorvível)</t>
+          <t>Aço inox 316L</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F138</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Metal biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>Clínico (Magmaris)</t>
+          <t>Clínico (1.ª geração)</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -18694,7 +18848,7 @@
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t>Revestimento de fármaco + polímero</t>
+          <t>Stent farmacológico → EtO (o fármaco limita)</t>
         </is>
       </c>
       <c r="N259" t="n">
@@ -18719,22 +18873,22 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>PLLA (bioabsorvível)</t>
+          <t>Co-Cr L605</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F90</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Polímero biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>Descontinuado (Absorb, 2017)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
@@ -18748,10 +18902,10 @@
         </is>
       </c>
       <c r="I260" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J260" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K260" t="inlineStr">
         <is>
@@ -18760,11 +18914,11 @@
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t>Gama degrada o PLLA (cisão de cadeias) → EtO obrigatório</t>
+          <t>Idem</t>
         </is>
       </c>
       <c r="N260" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O260" t="inlineStr">
         <is>
@@ -18785,12 +18939,12 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Aço inox 316L</t>
+          <t>Co-Ni-Cr-Mo MP35N</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>ASTM F138</t>
+          <t>ASTM F562</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
@@ -18800,12 +18954,12 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Clínico (1.ª geração)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -18814,23 +18968,23 @@
         </is>
       </c>
       <c r="I261" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J261" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K261" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t>Tecnologia de 1.ª geração</t>
+          <t>Idem</t>
         </is>
       </c>
       <c r="N261" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O261" t="inlineStr">
         <is>
@@ -18851,12 +19005,12 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Co-Cr L605</t>
+          <t>Pt-Cr</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>ASTM F90</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -18871,7 +19025,7 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
@@ -18880,18 +19034,23 @@
         </is>
       </c>
       <c r="I262" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J262" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>Idem</t>
         </is>
       </c>
       <c r="N262" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O262" t="inlineStr">
         <is>
@@ -18912,27 +19071,27 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Co-Ni-Cr-Mo MP35N</t>
+          <t>Nitinol (autoexpansível)</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>ASTM F562</t>
+          <t>ASTM F2063</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Metal (superelástico)</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Excluído (autoexpansível: só discussão)</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -18941,18 +19100,23 @@
         </is>
       </c>
       <c r="I263" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J263" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K263" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>Sem revestimento de fármaco (periférico)</t>
         </is>
       </c>
       <c r="N263" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O263" t="inlineStr">
         <is>
@@ -18973,7 +19137,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Pt-Cr</t>
+          <t>Liga de Mg WE43 (bioabsorvível)</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -18983,17 +19147,17 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Metal biodegradável</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Clínico (Magmaris)</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -19009,7 +19173,12 @@
       </c>
       <c r="K264" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>Revestimento de fármaco + polímero</t>
         </is>
       </c>
       <c r="N264" t="n">
@@ -19034,27 +19203,27 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Nitinol (autoexpansível)</t>
+          <t>PLLA (bioabsorvível)</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>ASTM F2063</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Metal (superelástico)</t>
+          <t>Polímero biodegradável</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Excluído (autoexpansível: só discussão)</t>
+          <t>Descontinuado (Absorb, 2017)</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
@@ -19063,18 +19232,23 @@
         </is>
       </c>
       <c r="I265" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J265" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K265" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>Gama degrada o PLLA (cisão de cadeias) → EtO obrigatório</t>
         </is>
       </c>
       <c r="N265" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O265" t="inlineStr">
         <is>
@@ -19095,22 +19269,22 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Liga de Mg WE43 (bioabsorvível)</t>
+          <t>Aço inox 316L</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F138</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Metal biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Clínico (Magmaris)</t>
+          <t>Clínico (1.ª geração)</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -19124,10 +19298,10 @@
         </is>
       </c>
       <c r="I266" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J266" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K266" t="inlineStr">
         <is>
@@ -19136,11 +19310,11 @@
       </c>
       <c r="M266" t="inlineStr">
         <is>
-          <t>Bioabsorvível</t>
+          <t>Tecnologia de 1.ª geração</t>
         </is>
       </c>
       <c r="N266" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
@@ -19161,22 +19335,22 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>PLLA (bioabsorvível)</t>
+          <t>Co-Cr L605</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F90</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Polímero biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Descontinuado (Absorb, 2017)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
@@ -19190,23 +19364,18 @@
         </is>
       </c>
       <c r="I267" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J267" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K267" t="inlineStr">
         <is>
           <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
-      <c r="M267" t="inlineStr">
-        <is>
-          <t>Bioabsorvível</t>
-        </is>
-      </c>
       <c r="N267" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O267" t="inlineStr">
         <is>
@@ -19227,12 +19396,12 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Aço inox 316L</t>
+          <t>Co-Ni-Cr-Mo MP35N</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>ASTM F138</t>
+          <t>ASTM F562</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
@@ -19242,12 +19411,12 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Clínico (1.ª geração)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>Fabricabilidade (ordinal 1-5)</t>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
@@ -19256,23 +19425,18 @@
         </is>
       </c>
       <c r="I268" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J268" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K268" t="inlineStr">
         <is>
-          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
-        </is>
-      </c>
-      <c r="M268" t="inlineStr">
-        <is>
-          <t>Corte laser de tubo maduro</t>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
       <c r="N268" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O268" t="inlineStr">
         <is>
@@ -19293,12 +19457,12 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Aço inox 316L</t>
+          <t>Pt-Cr</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>ASTM F138</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
@@ -19308,46 +19472,36 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Clínico (1.ª geração)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>Teor de níquel</t>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>% (massa)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I269" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J269" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="K269" t="inlineStr">
         <is>
-          <t>Página de fornecedor (Upmet), 316L ASTM F138</t>
-        </is>
-      </c>
-      <c r="L269" t="inlineStr">
-        <is>
-          <t>https://www.upmet.com/products/stainless-steel/316lslvm</t>
-        </is>
-      </c>
-      <c r="M269" t="inlineStr">
-        <is>
-          <t>fonte: página de fornecedor que declara cumprir a norma, não o texto da norma ASTM</t>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
       <c r="N269" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>Verificado (fornecedor)</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -19364,27 +19518,27 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Co-Cr L605</t>
+          <t>Nitinol (autoexpansível)</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>ASTM F90</t>
+          <t>ASTM F2063</t>
         </is>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Metal (superelástico)</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Excluído (autoexpansível: só discussão)</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>Fabricabilidade (ordinal 1-5)</t>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -19393,18 +19547,18 @@
         </is>
       </c>
       <c r="I270" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J270" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K270" t="inlineStr">
         <is>
-          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
       <c r="N270" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O270" t="inlineStr">
         <is>
@@ -19425,61 +19579,56 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Co-Cr L605</t>
+          <t>Liga de Mg WE43 (bioabsorvível)</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>ASTM F90</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Metal biodegradável</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Clínico (Magmaris)</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>Teor de níquel</t>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>% (massa)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I271" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J271" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>Página de fornecedor (MGM Industries), L605 ASTM F90</t>
-        </is>
-      </c>
-      <c r="L271" t="inlineStr">
-        <is>
-          <t>https://www.mgm-industries.com/l605-alloy</t>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t>fonte: página de fornecedor que declara cumprir a norma, não o texto da norma ASTM</t>
+          <t>Bioabsorvível</t>
         </is>
       </c>
       <c r="N271" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>Verificado (fornecedor)</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -19496,27 +19645,27 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Co-Ni-Cr-Mo MP35N</t>
+          <t>PLLA (bioabsorvível)</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>ASTM F562</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Metal</t>
+          <t>Polímero biodegradável</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Descontinuado (Absorb, 2017)</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>Fabricabilidade (ordinal 1-5)</t>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -19532,7 +19681,12 @@
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>Bioabsorvível</t>
         </is>
       </c>
       <c r="N272" t="n">
@@ -19557,12 +19711,12 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Co-Ni-Cr-Mo MP35N</t>
+          <t>Aço inox 316L</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>ASTM F562</t>
+          <t>ASTM F138</t>
         </is>
       </c>
       <c r="E273" t="inlineStr">
@@ -19572,46 +19726,41 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Clínico (1.ª geração)</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>Teor de níquel</t>
+          <t>Fabricabilidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>% (massa)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I273" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="J273" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="K273" t="inlineStr">
         <is>
-          <t>Página de fornecedor (stainless.eu), MP35N ASTM F562</t>
-        </is>
-      </c>
-      <c r="L273" t="inlineStr">
-        <is>
-          <t>https://www.stainless.eu/en/products/cobalt-alloys/mp35n/</t>
+          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
         <is>
-          <t>fonte: página de fornecedor que declara cumprir a norma, não o texto da norma ASTM</t>
+          <t>Corte laser de tubo maduro</t>
         </is>
       </c>
       <c r="N273" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>Verificado (fornecedor)</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -19628,12 +19777,12 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Pt-Cr</t>
+          <t>Aço inox 316L</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F138</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
@@ -19643,36 +19792,46 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>Clínico</t>
+          <t>Clínico (1.ª geração)</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>Fabricabilidade (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I274" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J274" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
+          <t>Página de fornecedor (Upmet), 316L ASTM F138</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>https://www.upmet.com/products/stainless-steel/316lslvm</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>fonte: página de fornecedor que declara cumprir a norma, não o texto da norma ASTM</t>
         </is>
       </c>
       <c r="N274" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -19689,12 +19848,12 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Pt-Cr</t>
+          <t>Co-Cr L605</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F90</t>
         </is>
       </c>
       <c r="E275" t="inlineStr">
@@ -19709,41 +19868,31 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>Teor de níquel</t>
+          <t>Fabricabilidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>% (massa)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I275" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J275" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t>A novel platinum chromium everolimus-eluting stent for the treatment of coronary artery disease. Biologics: Targets and Therapy 2013;7:149 [confirmar autores e ano]</t>
-        </is>
-      </c>
-      <c r="L275" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.2147/BTT.S34939</t>
-        </is>
-      </c>
-      <c r="M275" t="inlineStr">
-        <is>
-          <t>valor nominal, sem intervalo (PMC3692344: 33 % Fe, 33 % Pt, 18 % Cr, 9 % Ni, 3 % Mo)</t>
+          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
       <c r="N275" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -19760,56 +19909,61 @@
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Nitinol (autoexpansível)</t>
+          <t>Co-Cr L605</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>ASTM F2063</t>
+          <t>ASTM F90</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Metal (superelástico)</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Excluído (autoexpansível: só discussão)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>Fabricabilidade (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I276" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J276" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="K276" t="inlineStr">
         <is>
-          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
+          <t>Página de fornecedor (MGM Industries), L605 ASTM F90</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>https://www.mgm-industries.com/l605-alloy</t>
         </is>
       </c>
       <c r="M276" t="inlineStr">
         <is>
-          <t>Tratamento de memória de forma</t>
+          <t>fonte: página de fornecedor que declara cumprir a norma, não o texto da norma ASTM</t>
         </is>
       </c>
       <c r="N276" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -19826,22 +19980,22 @@
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Liga de Mg WE43 (bioabsorvível)</t>
+          <t>Co-Ni-Cr-Mo MP35N</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F562</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Metal biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Clínico (Magmaris)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -19855,23 +20009,18 @@
         </is>
       </c>
       <c r="I277" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J277" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K277" t="inlineStr">
         <is>
           <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
-      <c r="M277" t="inlineStr">
-        <is>
-          <t>Controlo de degradação e revestimentos</t>
-        </is>
-      </c>
       <c r="N277" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O277" t="inlineStr">
         <is>
@@ -19892,22 +20041,22 @@
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Liga de Mg WE43 (bioabsorvível)</t>
+          <t>Co-Ni-Cr-Mo MP35N</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F562</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Metal biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Clínico (Magmaris)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -19921,32 +20070,32 @@
         </is>
       </c>
       <c r="I278" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="J278" t="n">
-        <v>0.005</v>
+        <v>37</v>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t>MakeItFrom, WE43B (cita ASTM B80)</t>
+          <t>Página de fornecedor (stainless.eu), MP35N ASTM F562</t>
         </is>
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>https://www.makeitfrom.com/material-properties/WE43B-WE43B-T6-M18432-Magnesium</t>
+          <t>https://www.stainless.eu/en/products/cobalt-alloys/mp35n/</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
         <is>
-          <t>limite máximo de Ni como impureza; típico = máximo (pior caso); fonte secundária; a ficha Luxfer DS-467 (05/2026) não indica Ni; composição da liga do Magmaris não confirmada</t>
+          <t>fonte: página de fornecedor que declara cumprir a norma, não o texto da norma ASTM</t>
         </is>
       </c>
       <c r="N278" t="n">
-        <v>0.005</v>
+        <v>35</v>
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -19963,7 +20112,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>PLLA (bioabsorvível)</t>
+          <t>Pt-Cr</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -19973,12 +20122,12 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Polímero biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Descontinuado (Absorb, 2017)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -19992,23 +20141,18 @@
         </is>
       </c>
       <c r="I279" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J279" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K279" t="inlineStr">
         <is>
           <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
-      <c r="M279" t="inlineStr">
-        <is>
-          <t>Struts espessos; processamento térmico sensível</t>
-        </is>
-      </c>
       <c r="N279" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
@@ -20029,7 +20173,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>PLLA (bioabsorvível)</t>
+          <t>Pt-Cr</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -20039,12 +20183,12 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Polímero biodegradável</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Descontinuado (Absorb, 2017)</t>
+          <t>Clínico</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -20058,64 +20202,69 @@
         </is>
       </c>
       <c r="I280" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J280" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>Composição química do PLLA</t>
+          <t>A novel platinum chromium everolimus-eluting stent for the treatment of coronary artery disease. Biologics: Targets and Therapy 2013;7:149 [confirmar autores e ano]</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2147/BTT.S34939</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>polímero de C, H e O; sem metais</t>
+          <t>valor nominal, sem intervalo (PMC3692344: 33 % Fe, 33 % Pt, 18 % Cr, 9 % Ni, 3 % Mo)</t>
         </is>
       </c>
       <c r="N280" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>Verificado (composição química)</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>PCL</t>
+          <t>Nitinol (autoexpansível)</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ASTM F2063</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Metal (superelástico)</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>Clínico (uso limitado)</t>
+          <t>Excluído (autoexpansível: só discussão)</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Fabricabilidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H281" t="inlineStr">
@@ -20131,12 +20280,12 @@
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t>Fusão ~60 °C: sem autoclave; EtO/gama com cuidado; Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+          <t>Tratamento de memória de forma</t>
         </is>
       </c>
       <c r="N281" t="n">
@@ -20151,17 +20300,17 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>PLLA</t>
+          <t>Liga de Mg WE43 (bioabsorvível)</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -20171,17 +20320,17 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Metal biodegradável</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>Investigação</t>
+          <t>Clínico (Magmaris)</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Fabricabilidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
@@ -20197,12 +20346,12 @@
       </c>
       <c r="K282" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t>Gama causa cisão de cadeias; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+          <t>Controlo de degradação e revestimentos</t>
         </is>
       </c>
       <c r="N282" t="n">
@@ -20217,17 +20366,17 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>PLGA 50:50</t>
+          <t>Liga de Mg WE43 (bioabsorvível)</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -20237,68 +20386,68 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Metal biodegradável</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Investigação</t>
+          <t>Clínico (Magmaris)</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I283" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J283" t="n">
-        <v>2</v>
+        <v>0.005</v>
       </c>
       <c r="K283" t="inlineStr">
         <is>
-          <t>Holy CE, Cheng C, Davies JE, Shoichet MS. Biomaterials 2001;22:25-31 (Tabela 2)</t>
+          <t>MakeItFrom, WE43B (cita ASTM B80)</t>
         </is>
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/S0142-9612(00)00136-8</t>
+          <t>https://www.makeitfrom.com/material-properties/WE43B-WE43B-T6-M18432-Magnesium</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t>nota 2 pela rubrica (degradação documentada): gama 2,5 Mrad, Mw -54 %; EtO, Mw -12 % e volume -50 % (Holy 2001, texto completo); a fonte usa scaffolds de PLGA 75/25, não 50:50, e não indica a porosidade; Muito sensível: altera a degradação; Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+          <t>limite máximo de Ni como impureza; típico = máximo (pior caso); fonte secundária; a ficha Luxfer DS-467 (05/2026) não indica Ni; composição da liga do Magmaris não confirmada</t>
         </is>
       </c>
       <c r="N283" t="n">
-        <v>2</v>
+        <v>0.005</v>
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Hidroxiapatite (HA) porosa</t>
+          <t>PLLA (bioabsorvível)</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -20308,17 +20457,17 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Cerâmico</t>
+          <t>Polímero biodegradável</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo)</t>
+          <t>Descontinuado (Absorb, 2017)</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Fabricabilidade (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
@@ -20327,23 +20476,23 @@
         </is>
       </c>
       <c r="I284" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J284" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K284" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Geetha 2009; Navarro 2008; literatura de fabrico aditivo: confirmar</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>a confirmar: o autoclave (121 °C, 40 min) altera a dissolubilidade, a resistência e a morfologia da HA porosa (Li X et al. J Mater Sci Mater Med 2016;27:5, https://doi.org/10.1007/s10856-015-5617-x, só resumo); falta fonte para radiação gama em HA; Autoclave/calor seco; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>Struts espessos; processamento térmico sensível</t>
         </is>
       </c>
       <c r="N284" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O284" t="inlineStr">
         <is>
@@ -20354,17 +20503,17 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Scaffold (regeneração óssea)</t>
+          <t>Stent vascular</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Scaffold poroso</t>
+          <t>Estrutura do stent</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>β-TCP poroso</t>
+          <t>PLLA (bioabsorvível)</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -20374,51 +20523,46 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Cerâmico</t>
+          <t>Polímero biodegradável</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo)</t>
+          <t>Descontinuado (Absorb, 2017)</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
+          <t>Teor de níquel</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>% (massa)</t>
         </is>
       </c>
       <c r="I285" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J285" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K285" t="inlineStr">
         <is>
-          <t>FDA 510(k) K032409 (Vitoss, Orthovita, 2003); FDA 510(k) K120152 (Cerasorb Plus, Riemser, 2012)</t>
-        </is>
-      </c>
-      <c r="L285" t="inlineStr">
-        <is>
-          <t>https://fda.innolitics.com/device/K032409</t>
+          <t>Composição química do PLLA</t>
         </is>
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t>nota 5 pela rubrica: os dois produtos são esterilizados por radiação gama (resumos dos 510(k), lidos numa cópia de terceiros, https://fda.innolitics.com/device/K120152); ressalva: o autoclave altera a morfologia e a resistência do β-TCP poroso (Li X et al. J Mater Sci Mater Med 2016;27:5, https://doi.org/10.1007/s10856-015-5617-x, só resumo); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>polímero de C, H e O; sem metais</t>
         </is>
       </c>
       <c r="N285" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>Verificado (fornecedor)</t>
+          <t>Verificado (composição química)</t>
         </is>
       </c>
     </row>
@@ -20435,7 +20579,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Vidro bioativo 45S5 poroso</t>
+          <t>PCL</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -20445,12 +20589,12 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Vidro</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo, partículas)</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
@@ -20464,10 +20608,10 @@
         </is>
       </c>
       <c r="I286" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J286" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K286" t="inlineStr">
         <is>
@@ -20476,11 +20620,11 @@
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t>calor seco; a radiação gama aumenta a dissolução (Farag 2017, só resumo, https://doi.org/10.1002/jbm.a.36035); Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+          <t>Fusão ~60 °C: sem autoclave; EtO/gama com cuidado; Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
         </is>
       </c>
       <c r="N286" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O286" t="inlineStr">
         <is>
@@ -20501,7 +20645,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Compósito PCL/β-TCP (impressão 3D)</t>
+          <t>PLLA</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -20511,12 +20655,12 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Compósito</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>Clínico (uso limitado)</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -20537,17 +20681,12 @@
       </c>
       <c r="K287" t="inlineStr">
         <is>
-          <t>Bruyas A et al. Tissue Eng Part A 2019;25:248-256</t>
-        </is>
-      </c>
-      <c r="L287" t="inlineStr">
-        <is>
-          <t>https://doi.org/10.1089/ten.tea.2018.0130</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t>nota 3 pela rubrica (método restrito com risco de degradação): scaffolds PCL/β-TCP por FDM, feixe de eletrões: +14 % de rigidez e resistência iniciais e degradação 25 % mais rápida (Bruyas 2019, só resumo); o calor está excluído pela fusão do PCL; Limitado pela fase PCL; Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>Gama causa cisão de cadeias; Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N287" t="n">
@@ -20555,7 +20694,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -20572,7 +20711,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Quitosano/HA (liofilizado)</t>
+          <t>PLGA 50:50</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -20582,7 +20721,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Compósito natural</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -20601,27 +20740,32 @@
         </is>
       </c>
       <c r="I288" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J288" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K288" t="inlineStr">
         <is>
-          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
+          <t>Holy CE, Cheng C, Davies JE, Shoichet MS. Biomaterials 2001;22:25-31 (Tabela 2)</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/S0142-9612(00)00136-8</t>
         </is>
       </c>
       <c r="M288" t="inlineStr">
         <is>
-          <t>Polímero natural sensível ao calor; Estatuto [confirmar]: fonte a indicar</t>
+          <t>nota 2 pela rubrica (degradação documentada): gama 2,5 Mrad, Mw -54 %; EtO, Mw -12 % e volume -50 % (Holy 2001, texto completo); a fonte usa scaffolds de PLGA 75/25, não 50:50, e não indica a porosidade; Muito sensível: altera a degradação; Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
         </is>
       </c>
       <c r="N288" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -20638,7 +20782,7 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>PCL</t>
+          <t>Hidroxiapatite (HA) porosa</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -20648,17 +20792,17 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Cerâmico</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Clínico (uso limitado)</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
@@ -20667,23 +20811,23 @@
         </is>
       </c>
       <c r="I289" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J289" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K289" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M289" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
+          <t>a confirmar: o autoclave (121 °C, 40 min) altera a dissolubilidade, a resistência e a morfologia da HA porosa (Li X et al. J Mater Sci Mater Med 2016;27:5, https://doi.org/10.1007/s10856-015-5617-x, só resumo); falta fonte para radiação gama em HA; Autoclave/calor seco; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N289" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O289" t="inlineStr">
         <is>
@@ -20704,7 +20848,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>PLLA</t>
+          <t>β-TCP poroso</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -20714,17 +20858,17 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Cerâmico</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>Investigação</t>
+          <t>Clínico (substituto ósseo)</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H290" t="inlineStr">
@@ -20733,27 +20877,32 @@
         </is>
       </c>
       <c r="I290" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J290" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K290" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>FDA 510(k) K032409 (Vitoss, Orthovita, 2003); FDA 510(k) K120152 (Cerasorb Plus, Riemser, 2012)</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>https://fda.innolitics.com/device/K032409</t>
         </is>
       </c>
       <c r="M290" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
+          <t>nota 5 pela rubrica: os dois produtos são esterilizados por radiação gama (resumos dos 510(k), lidos numa cópia de terceiros, https://fda.innolitics.com/device/K120152); ressalva: o autoclave altera a morfologia e a resistência do β-TCP poroso (Li X et al. J Mater Sci Mater Med 2016;27:5, https://doi.org/10.1007/s10856-015-5617-x, só resumo); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N290" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -20770,7 +20919,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>PLGA 50:50</t>
+          <t>Vidro bioativo 45S5 poroso</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -20780,17 +20929,17 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Polímero</t>
+          <t>Vidro</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>Investigação</t>
+          <t>Clínico (substituto ósseo, partículas)</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
@@ -20799,23 +20948,23 @@
         </is>
       </c>
       <c r="I291" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J291" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K291" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M291" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
+          <t>calor seco; a radiação gama aumenta a dissolução (Farag 2017, só resumo, https://doi.org/10.1002/jbm.a.36035); Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
         </is>
       </c>
       <c r="N291" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O291" t="inlineStr">
         <is>
@@ -20836,7 +20985,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Hidroxiapatite (HA) porosa</t>
+          <t>Compósito PCL/β-TCP (impressão 3D)</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -20846,17 +20995,17 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Cerâmico</t>
+          <t>Compósito</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo)</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H292" t="inlineStr">
@@ -20872,12 +21021,17 @@
       </c>
       <c r="K292" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>Bruyas A et al. Tissue Eng Part A 2019;25:248-256</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1089/ten.tea.2018.0130</t>
         </is>
       </c>
       <c r="M292" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>nota 3 pela rubrica (método restrito com risco de degradação): scaffolds PCL/β-TCP por FDM, feixe de eletrões: +14 % de rigidez e resistência iniciais e degradação 25 % mais rápida (Bruyas 2019, só resumo); o calor está excluído pela fusão do PCL; Limitado pela fase PCL; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N292" t="n">
@@ -20885,7 +21039,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -20902,7 +21056,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>β-TCP poroso</t>
+          <t>Quitosano/HA (liofilizado)</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -20912,17 +21066,17 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Cerâmico</t>
+          <t>Compósito natural</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo)</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+          <t>Compatibilidade com esterilização (ordinal 1-5)</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
@@ -20938,12 +21092,12 @@
       </c>
       <c r="K293" t="inlineStr">
         <is>
-          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+          <t>ISO 11137 (radiação) / ISO 11135 (EtO); Kurtz 2016 para UHMWPE: confirmar</t>
         </is>
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>Polímero natural sensível ao calor; Estatuto [confirmar]: fonte a indicar</t>
         </is>
       </c>
       <c r="N293" t="n">
@@ -20968,7 +21122,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Vidro bioativo 45S5 poroso</t>
+          <t>PCL</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -20978,12 +21132,12 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Vidro</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Clínico (substituto ósseo, partículas)</t>
+          <t>Clínico (uso limitado)</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -20997,10 +21151,10 @@
         </is>
       </c>
       <c r="I294" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J294" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K294" t="inlineStr">
         <is>
@@ -21009,11 +21163,11 @@
       </c>
       <c r="M294" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+          <t>Estatuto [confirmar]: Woodruff &amp; Hutmacher 2010</t>
         </is>
       </c>
       <c r="N294" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O294" t="inlineStr">
         <is>
@@ -21034,7 +21188,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Compósito PCL/β-TCP (impressão 3D)</t>
+          <t>PLLA</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -21044,12 +21198,12 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Compósito</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>Clínico (uso limitado)</t>
+          <t>Investigação</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
@@ -21063,10 +21217,10 @@
         </is>
       </c>
       <c r="I295" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J295" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K295" t="inlineStr">
         <is>
@@ -21075,11 +21229,11 @@
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; uso clínico noutras formas (fixação)</t>
         </is>
       </c>
       <c r="N295" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O295" t="inlineStr">
         <is>
@@ -21100,7 +21254,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Quitosano/HA (liofilizado)</t>
+          <t>PLGA 50:50</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -21110,7 +21264,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Compósito natural</t>
+          <t>Polímero</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -21141,7 +21295,7 @@
       </c>
       <c r="M296" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: fonte a indicar</t>
+          <t>Estatuto [confirmar]: Athanasiou et al. 1996; uso clínico noutras formas</t>
         </is>
       </c>
       <c r="N296" t="n">
@@ -21153,8 +21307,338 @@
         </is>
       </c>
     </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Hidroxiapatite (HA) porosa</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Cerâmico</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Clínico (substituto ósseo)</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>3</v>
+      </c>
+      <c r="J297" t="n">
+        <v>3</v>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
+      <c r="N297" t="n">
+        <v>3</v>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>β-TCP poroso</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Cerâmico</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Clínico (substituto ósseo)</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>3</v>
+      </c>
+      <c r="J298" t="n">
+        <v>3</v>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+        </is>
+      </c>
+      <c r="N298" t="n">
+        <v>3</v>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Vidro bioativo 45S5 poroso</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Vidro</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Clínico (substituto ósseo, partículas)</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>4</v>
+      </c>
+      <c r="J299" t="n">
+        <v>4</v>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: Hench 1991; scaffold poroso sobretudo investigação</t>
+        </is>
+      </c>
+      <c r="N299" t="n">
+        <v>4</v>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Compósito PCL/β-TCP (impressão 3D)</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Compósito</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Clínico (uso limitado)</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>2</v>
+      </c>
+      <c r="J300" t="n">
+        <v>2</v>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte clínica a indicar</t>
+        </is>
+      </c>
+      <c r="N300" t="n">
+        <v>2</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Scaffold (regeneração óssea)</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Scaffold poroso</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Quitosano/HA (liofilizado)</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Compósito natural</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Investigação</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Custo relativo de material e fabrico (1-5, 5 = mais caro)</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>2</v>
+      </c>
+      <c r="J301" t="n">
+        <v>2</v>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>Índice relativo de material e fabrico (rubrica no LEIA-ME); não representa preço hospitalar</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>Estatuto [confirmar]: fonte a indicar</t>
+        </is>
+      </c>
+      <c r="N301" t="n">
+        <v>2</v>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>A verificar</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P296"/>
+  <autoFilter ref="A1:P301"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21814,7 +22298,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -21890,7 +22374,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Estética (ordinal 1-5)</t>
+          <t>Resistência à corrosão em meio oral (ordinal 1-5)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -21908,7 +22392,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Sombra cinzenta em gengiva fina</t>
+          <t>Problema crítico do docente (2 out 2026): fluoretos em meio ácido, tribocorrosão na ligação implante-pilar, envelhecimento da Y-TZP</t>
         </is>
       </c>
     </row>
@@ -21920,21 +22404,26 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Densidade</t>
+          <t>Estética (ordinal 1-5)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Custo</t>
+          <t>Benefício</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>g/cm³</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Sombra cinzenta em gengiva fina</t>
+        </is>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
Scaffold: Wang 2024 retirado do módulo do PCL/β-TCP (Editor Note da revista por esclarecer)
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -13314,7 +13314,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>regra da porosidade (típico do PCL/β-TCP: 70 %, janela 60-80 %), PCL/TCP 80:20 por FDM ou extrusão: a verificar, duas fontes fracas: 2,2 MPa a 59,5 %, no limite inferior da janela (Kawai 2018, texto completo); 6,38 MPa a 70 % (Wong 2025, fonte secundária, https://doi.org/10.7759/cureus.86272); típico = ponto médio; de fora: 27,9 MPa em Wang 2024, que não é tensão de cedência; valor anterior: 3-12 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>regra da porosidade (típico do PCL/β-TCP: 70 %, janela 60-80 %), PCL/TCP 80:20 por FDM ou extrusão: a verificar, duas fontes fracas: 2,2 MPa a 59,5 %, no limite inferior da janela (Kawai 2018, texto completo); 6,38 MPa a 70 % (Wong 2025, fonte secundária, https://doi.org/10.7759/cureus.86272); típico = ponto médio; de fora: 27,9 MPa em Wang 2024, que não é tensão de cedência (o Wang 2024 foi retirado de toda a base a 3 out 2026: Editor Note da revista, ver o módulo); valor anterior: 3-12 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N175" t="n">
@@ -13375,7 +13375,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>Reichert JC et al. Int Orthop 2011;35:1229-1236; Wang Y et al. Heliyon 2024;10:e26071 (Tabela 3); Kawai T et al. J Orthop Res 2018;36:1002-1011</t>
+          <t>Reichert JC et al. Int Orthop 2011;35:1229-1236; Kawai T et al. J Orthop Res 2018;36:1002-1011</t>
         </is>
       </c>
       <c r="L176" t="inlineStr">
@@ -13385,11 +13385,11 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>regra da porosidade (típico do PCL/β-TCP: 70 %, janela 60-80 %), PCL/TCP 80:20 por FDM ou extrusão, típico = mediana de quatro valores: 22,2 MPa a 70,6 % em PBS (Reichert 2011, mPCL-TCP); 48,2 MPa a 65,1 % (Wang 2024, https://doi.org/10.1016/j.heliyon.2024.e26071); 51,5 MPa a 59,5 % (Kawai 2018, https://doi.org/10.1002/jor.23673); 23,1 MPa a 70 % (Wong 2025, fonte secundária, https://doi.org/10.7759/cureus.86272); texto completo em todas; valor anterior: 30-150 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>regra da porosidade (típico do PCL/β-TCP: 70 %, janela 60-80 %), PCL/TCP 80:20 por FDM ou extrusão, típico = mediana de três valores: 22,2 MPa a 70,6 % em PBS (Reichert 2011, mPCL-TCP); 51,5 MPa a 59,5 % (Kawai 2018, https://doi.org/10.1002/jor.23673); 23,1 MPa a 70 % (Wong 2025, fonte secundária, https://doi.org/10.7759/cureus.86272); texto completo em todas; retirado a 3 out 2026: 48,2 MPa a 65,1 % (Wang Y et al. Heliyon 2024;10:e26071), porque a revista publicou uma Editor Note sobre o artigo (doi:10.1016/j.heliyon.2025.e44205) cujo conteúdo não foi possível confirmar, e a Tabela 3 dá uma resistência (27,9 MPa) quase igual ao módulo (48,2 MPa), pouco plausível num scaffold poroso; típico anterior: 35,7 MPa (mediana de quatro valores); valor anterior: 30-150 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N176" t="n">
-        <v>35.7</v>
+        <v>23.1</v>
       </c>
       <c r="O176" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Relatório, etapa 3: cenário de teto de orçamento, consenso de Borda e anexos A e B
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -23550,7 +23550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -23791,6 +23791,23 @@
         </is>
       </c>
       <c r="C14" t="inlineStr">
+        <is>
+          <t>Todos os quantitativos</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>O-orçamento</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Teto de orçamento: exclui na triagem os materiais com custo relativo acima de teto_custo_relativo (3), sem mudar os pesos; cenário A</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>Todos os quantitativos</t>
         </is>
@@ -24153,7 +24170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -24223,6 +24240,21 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>teto_custo_relativo</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Cenário O-orçamento: exclui na triagem os materiais com custo relativo de material e fabrico (ordinal 1-5) acima deste valor, sem mudar os pesos; casos quantitativos, cenário A; valor de desenho</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Relatório, versão 1: fontes das 16 marcas e das 3 da base, 12 referências novas, anexo B resumido e figuras sem arredondar para 100 %
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -2156,27 +2156,27 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>7.9</v>
+        <v>8</v>
       </c>
       <c r="J6" t="n">
         <v>8</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>[fonte a indicar] (o Niinomi 1998 é só de ligas de Ti)</t>
+          <t>Alleima, ficha 316LVM</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Valores dependem muito de recozido vs encruado</t>
+          <t>mesma ficha da linha do stent (Alleima 316LVM, 8,0 g/cm³); a densidade não depende do encruamento de forma relevante; ficha da Alleima sem URL registado; valor anterior: 7,9-8,0 g/cm³ [sem fonte]; Valores dependem muito de recozido vs encruado (nota antiga, válida para as propriedades mecânicas)</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>7.95</v>
+        <v>8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -2567,27 +2567,32 @@
         </is>
       </c>
       <c r="I12" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="J12" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="J12" t="n">
-        <v>8.5</v>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>[fonte a indicar] (o Niinomi 1998 é só de ligas de Ti)</t>
+          <t>Alleima, ficha Alleima F1537 (barra); Fort Wayne Metals, FWM 1537 alloy</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.alleima.com/en/technical-center/material-datasheets/bar-and-hollow-bar/bar/alleima-f1537/</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Slides: F799 ~2x fadiga/cedência da F75</t>
+          <t>mín.: 8,25 g/cm³ a 20 °C (Alleima F1537, barra, ficha de 12 nov 2025); máx.: 8,30 g/cm³ (Fort Wayne Metals, FWM 1537, https://fwmetals.com/what-we-do/materials/high-performance-alloys/fwm-1537-alloy); típico = ponto médio; a ASTM F1537 não define a densidade; valor anterior: 8,3-8,5 g/cm³ [sem fonte]; Slides: F799 ~2x fadiga/cedência da F75</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>8.4</v>
+        <v>8.275</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado (fornecedor)</t>
         </is>
       </c>
     </row>
@@ -20209,7 +20214,7 @@
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>A novel platinum chromium everolimus-eluting stent for the treatment of coronary artery disease. Biologics: Targets and Therapy 2013;7:149 [confirmar autores e ano]</t>
+          <t>Bennett J, Dubois C. A novel platinum chromium everolimus-eluting stent for the treatment of coronary artery disease. Biologics 2013;7:149-159</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
@@ -20219,7 +20224,7 @@
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>valor nominal, sem intervalo (PMC3692344: 33 % Fe, 33 % Pt, 18 % Cr, 9 % Ni, 3 % Mo)</t>
+          <t>valor nominal, sem intervalo (PMC3692344: 33 % Fe, 33 % Pt, 18 % Cr, 9 % Ni, 3 % Mo); autores pela ordem do PubMed (PMID 23818756; a Crossref inverte a ordem)</t>
         </is>
       </c>
       <c r="N280" t="n">

</xml_diff>